<commit_message>
HOME BASE: finally was able to reproduce some of the trends from the original spreadsheet
</commit_message>
<xml_diff>
--- a/results/validate_results.xlsx
+++ b/results/validate_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emily/Library/CloudStorage/GoogleDrive-u0835353@gcloud.utah.edu/.shortcut-targets-by-id/109kT4myKnMujFK8ni-DWM3IQ1FnMmvXr/EYANG/BCI Project/FWHT_FeatureExtract/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2237F3C4-479B-3A47-9B47-F993D5CFA83E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9BFF027-49AE-374A-8306-7D33631513DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-22140" yWindow="-21120" windowWidth="38400" windowHeight="21120" xr2:uid="{AFAE147A-AF5E-4547-B045-936377B9E7D9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="46">
   <si>
     <t>Easy1</t>
   </si>
@@ -171,6 +171,9 @@
   </si>
   <si>
     <t>kmeans_window.m inside 2026_04_21</t>
+  </si>
+  <si>
+    <t>Euclidean</t>
   </si>
 </sst>
 </file>
@@ -313,7 +316,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
@@ -360,6 +363,10 @@
     <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -705,6 +712,11 @@
         <v>44</v>
       </c>
     </row>
+    <row r="2" spans="3:28" x14ac:dyDescent="0.2">
+      <c r="C2" t="s">
+        <v>45</v>
+      </c>
+    </row>
     <row r="3" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C3" s="14" t="s">
         <v>35</v>
@@ -828,32 +840,48 @@
       <c r="K5" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="L5" s="22"/>
-      <c r="M5" s="23"/>
+      <c r="L5" s="22">
+        <v>98.574854454457494</v>
+      </c>
+      <c r="M5" s="23">
+        <v>97.43</v>
+      </c>
       <c r="O5" s="21" t="s">
         <v>0</v>
       </c>
       <c r="P5" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="Q5" s="22"/>
-      <c r="R5" s="23"/>
+      <c r="Q5" s="22">
+        <v>99.002890240902701</v>
+      </c>
+      <c r="R5" s="23">
+        <v>97.57</v>
+      </c>
       <c r="T5" s="21" t="s">
         <v>0</v>
       </c>
       <c r="U5" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="V5" s="22"/>
-      <c r="W5" s="23"/>
+      <c r="V5" s="36">
+        <v>99.002890240902701</v>
+      </c>
+      <c r="W5" s="23">
+        <v>97.86</v>
+      </c>
       <c r="Y5" s="8" t="s">
         <v>0</v>
       </c>
       <c r="Z5" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="AA5" s="9"/>
-      <c r="AB5" s="10"/>
+      <c r="AA5" s="34">
+        <v>99.148302585035395</v>
+      </c>
+      <c r="AB5" s="10">
+        <v>98.01</v>
+      </c>
     </row>
     <row r="6" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C6" s="21"/>
@@ -876,26 +904,42 @@
       <c r="K6" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="L6" s="22"/>
-      <c r="M6" s="23"/>
+      <c r="L6" s="22">
+        <v>98.577017107872706</v>
+      </c>
+      <c r="M6" s="23">
+        <v>96.76</v>
+      </c>
       <c r="O6" s="21"/>
       <c r="P6" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="Q6" s="22"/>
-      <c r="R6" s="23"/>
+      <c r="Q6" s="22">
+        <v>98.687480598085301</v>
+      </c>
+      <c r="R6" s="23">
+        <v>97.04</v>
+      </c>
       <c r="T6" s="21"/>
       <c r="U6" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="V6" s="22"/>
-      <c r="W6" s="23"/>
+      <c r="V6" s="36">
+        <v>99.563480747068098</v>
+      </c>
+      <c r="W6" s="23">
+        <v>97.04</v>
+      </c>
       <c r="Y6" s="8"/>
       <c r="Z6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="AA6" s="9"/>
-      <c r="AB6" s="10"/>
+      <c r="AA6" s="34">
+        <v>99.454557622808196</v>
+      </c>
+      <c r="AB6" s="10">
+        <v>97.03</v>
+      </c>
     </row>
     <row r="7" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C7" s="21"/>
@@ -918,26 +962,42 @@
       <c r="K7" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="L7" s="22"/>
-      <c r="M7" s="23"/>
+      <c r="L7" s="22">
+        <v>98.6800879070761</v>
+      </c>
+      <c r="M7" s="23">
+        <v>97.06</v>
+      </c>
       <c r="O7" s="21"/>
       <c r="P7" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="Q7" s="22"/>
-      <c r="R7" s="23"/>
+      <c r="Q7" s="22">
+        <v>99.263354797323302</v>
+      </c>
+      <c r="R7" s="23">
+        <v>96.73</v>
+      </c>
       <c r="T7" s="21"/>
       <c r="U7" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="V7" s="22"/>
-      <c r="W7" s="23"/>
+      <c r="V7" s="36">
+        <v>99.263354797323302</v>
+      </c>
+      <c r="W7" s="23">
+        <v>96.73</v>
+      </c>
       <c r="Y7" s="8"/>
       <c r="Z7" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="AA7" s="9"/>
-      <c r="AB7" s="10"/>
+      <c r="AA7" s="34">
+        <v>99.413444199559194</v>
+      </c>
+      <c r="AB7" s="10">
+        <v>96.73</v>
+      </c>
     </row>
     <row r="8" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C8" s="21"/>
@@ -960,26 +1020,42 @@
       <c r="K8" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="L8" s="22"/>
-      <c r="M8" s="23"/>
+      <c r="L8" s="22">
+        <v>97.531177473946698</v>
+      </c>
+      <c r="M8" s="23">
+        <v>95.52</v>
+      </c>
       <c r="O8" s="21"/>
       <c r="P8" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="Q8" s="22"/>
-      <c r="R8" s="23"/>
+      <c r="Q8" s="22">
+        <v>97.985950453055693</v>
+      </c>
+      <c r="R8" s="23">
+        <v>96.54</v>
+      </c>
       <c r="T8" s="21"/>
       <c r="U8" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="V8" s="22"/>
-      <c r="W8" s="23"/>
+      <c r="V8" s="36">
+        <v>98.986707472223003</v>
+      </c>
+      <c r="W8" s="23">
+        <v>96.54</v>
+      </c>
       <c r="Y8" s="8"/>
       <c r="Z8" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="AA8" s="9"/>
-      <c r="AB8" s="10"/>
+      <c r="AA8" s="34">
+        <v>98.856727876335697</v>
+      </c>
+      <c r="AB8" s="10">
+        <v>96.55</v>
+      </c>
     </row>
     <row r="9" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C9" s="21"/>
@@ -1002,26 +1078,42 @@
       <c r="K9" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="L9" s="22"/>
-      <c r="M9" s="23"/>
+      <c r="L9" s="22">
+        <v>98.633530623712701</v>
+      </c>
+      <c r="M9" s="23">
+        <v>97.11</v>
+      </c>
       <c r="O9" s="21"/>
       <c r="P9" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="Q9" s="22"/>
-      <c r="R9" s="23"/>
+      <c r="Q9" s="22">
+        <v>99.086401427689395</v>
+      </c>
+      <c r="R9" s="23">
+        <v>97.42</v>
+      </c>
       <c r="T9" s="21"/>
       <c r="U9" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="V9" s="22"/>
-      <c r="W9" s="23"/>
+      <c r="V9" s="36">
+        <v>99.395047491992898</v>
+      </c>
+      <c r="W9" s="23">
+        <v>97.42</v>
+      </c>
       <c r="Y9" s="8"/>
       <c r="Z9" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="AA9" s="9"/>
-      <c r="AB9" s="10"/>
+      <c r="AA9" s="34">
+        <v>99.695824357606298</v>
+      </c>
+      <c r="AB9" s="10">
+        <v>97.27</v>
+      </c>
     </row>
     <row r="10" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C10" s="21"/>
@@ -1044,26 +1136,42 @@
       <c r="K10" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="L10" s="22"/>
-      <c r="M10" s="23"/>
+      <c r="L10" s="22">
+        <v>97.541939235450499</v>
+      </c>
+      <c r="M10" s="23">
+        <v>94.81</v>
+      </c>
       <c r="O10" s="21"/>
       <c r="P10" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="Q10" s="22"/>
-      <c r="R10" s="23"/>
+      <c r="Q10" s="22">
+        <v>98.269193690481302</v>
+      </c>
+      <c r="R10" s="23">
+        <v>95.09</v>
+      </c>
       <c r="T10" s="21"/>
       <c r="U10" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="V10" s="22"/>
-      <c r="W10" s="23"/>
+      <c r="V10" s="36">
+        <v>98.984456578837296</v>
+      </c>
+      <c r="W10" s="23">
+        <v>95.09</v>
+      </c>
       <c r="Y10" s="8"/>
       <c r="Z10" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="AA10" s="9"/>
-      <c r="AB10" s="10"/>
+      <c r="AA10" s="34">
+        <v>99.275177048739906</v>
+      </c>
+      <c r="AB10" s="10">
+        <v>94.81</v>
+      </c>
     </row>
     <row r="11" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C11" s="21"/>
@@ -1086,26 +1194,42 @@
       <c r="K11" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="L11" s="22"/>
-      <c r="M11" s="23"/>
+      <c r="L11" s="22">
+        <v>97.476847073323299</v>
+      </c>
+      <c r="M11" s="23">
+        <v>94.53</v>
+      </c>
       <c r="O11" s="21"/>
       <c r="P11" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="Q11" s="22"/>
-      <c r="R11" s="23"/>
+      <c r="Q11" s="22">
+        <v>97.900520199457105</v>
+      </c>
+      <c r="R11" s="23">
+        <v>93.81</v>
+      </c>
       <c r="T11" s="21"/>
       <c r="U11" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="V11" s="22"/>
-      <c r="W11" s="23"/>
+      <c r="V11" s="36">
+        <v>98.606619399039701</v>
+      </c>
+      <c r="W11" s="23">
+        <v>93.81</v>
+      </c>
       <c r="Y11" s="8"/>
       <c r="Z11" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="AA11" s="9"/>
-      <c r="AB11" s="10"/>
+      <c r="AA11" s="34">
+        <v>98.877563424654994</v>
+      </c>
+      <c r="AB11" s="10">
+        <v>93.4</v>
+      </c>
     </row>
     <row r="12" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C12" s="21"/>
@@ -1128,26 +1252,42 @@
       <c r="K12" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="L12" s="22"/>
-      <c r="M12" s="23"/>
+      <c r="L12" s="22">
+        <v>97.977486929353006</v>
+      </c>
+      <c r="M12" s="23">
+        <v>94.66</v>
+      </c>
       <c r="O12" s="21"/>
       <c r="P12" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="Q12" s="22"/>
-      <c r="R12" s="23"/>
+      <c r="Q12" s="22">
+        <v>98.120668126227201</v>
+      </c>
+      <c r="R12" s="23">
+        <v>92.19</v>
+      </c>
       <c r="T12" s="21"/>
       <c r="U12" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="V12" s="22"/>
-      <c r="W12" s="23"/>
+      <c r="V12" s="36">
+        <v>98.554234247398796</v>
+      </c>
+      <c r="W12" s="23">
+        <v>92.34</v>
+      </c>
       <c r="Y12" s="8"/>
       <c r="Z12" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="AA12" s="9"/>
-      <c r="AB12" s="10"/>
+      <c r="AA12" s="34">
+        <v>98.699674706335301</v>
+      </c>
+      <c r="AB12" s="10">
+        <v>90.6</v>
+      </c>
     </row>
     <row r="13" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C13" s="21" t="s">
@@ -1174,32 +1314,48 @@
       <c r="K13" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="L13" s="22"/>
-      <c r="M13" s="23"/>
+      <c r="L13" s="22">
+        <v>98.376931659705093</v>
+      </c>
+      <c r="M13" s="23">
+        <v>95.85</v>
+      </c>
       <c r="O13" s="21" t="s">
         <v>9</v>
       </c>
       <c r="P13" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="Q13" s="22"/>
-      <c r="R13" s="23"/>
+      <c r="Q13" s="22">
+        <v>98.378796537364295</v>
+      </c>
+      <c r="R13" s="23">
+        <v>95.85</v>
+      </c>
       <c r="T13" s="21" t="s">
         <v>9</v>
       </c>
       <c r="U13" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="V13" s="22"/>
-      <c r="W13" s="23"/>
+      <c r="V13" s="36">
+        <v>98.686403838798796</v>
+      </c>
+      <c r="W13" s="23">
+        <v>97.05</v>
+      </c>
       <c r="Y13" s="8" t="s">
         <v>9</v>
       </c>
       <c r="Z13" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="AA13" s="9"/>
-      <c r="AB13" s="10"/>
+      <c r="AA13" s="34">
+        <v>98.977735045550403</v>
+      </c>
+      <c r="AB13" s="10">
+        <v>97.2</v>
+      </c>
     </row>
     <row r="14" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C14" s="21"/>
@@ -1222,26 +1378,42 @@
       <c r="K14" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="L14" s="22"/>
-      <c r="M14" s="23"/>
+      <c r="L14" s="22">
+        <v>97.088563433336503</v>
+      </c>
+      <c r="M14" s="23">
+        <v>92.9</v>
+      </c>
       <c r="O14" s="21"/>
       <c r="P14" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="Q14" s="22"/>
-      <c r="R14" s="23"/>
+      <c r="Q14" s="22">
+        <v>98.064103972194403</v>
+      </c>
+      <c r="R14" s="23">
+        <v>93.47</v>
+      </c>
       <c r="T14" s="21"/>
       <c r="U14" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="V14" s="22"/>
-      <c r="W14" s="23"/>
+      <c r="V14" s="36">
+        <v>98.748524920891498</v>
+      </c>
+      <c r="W14" s="23">
+        <v>93.47</v>
+      </c>
       <c r="Y14" s="8"/>
       <c r="Z14" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="AA14" s="9"/>
-      <c r="AB14" s="10"/>
+      <c r="AA14" s="34">
+        <v>99.020127901968905</v>
+      </c>
+      <c r="AB14" s="10">
+        <v>93.47</v>
+      </c>
     </row>
     <row r="15" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C15" s="21" t="s">
@@ -1268,32 +1440,48 @@
       <c r="K15" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="L15" s="22"/>
-      <c r="M15" s="23"/>
+      <c r="L15" s="22">
+        <v>96.350895844665303</v>
+      </c>
+      <c r="M15" s="23">
+        <v>91.39</v>
+      </c>
       <c r="O15" s="21" t="s">
         <v>10</v>
       </c>
       <c r="P15" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="Q15" s="22"/>
-      <c r="R15" s="23"/>
+      <c r="Q15" s="22">
+        <v>97.235785607012502</v>
+      </c>
+      <c r="R15" s="23">
+        <v>92.12</v>
+      </c>
       <c r="T15" s="21" t="s">
         <v>10</v>
       </c>
       <c r="U15" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="V15" s="22"/>
-      <c r="W15" s="23"/>
+      <c r="V15" s="36">
+        <v>97.5323644666679</v>
+      </c>
+      <c r="W15" s="23">
+        <v>92.12</v>
+      </c>
       <c r="Y15" s="8" t="s">
         <v>10</v>
       </c>
       <c r="Z15" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="AA15" s="9"/>
-      <c r="AB15" s="10"/>
+      <c r="AA15" s="34">
+        <v>98.405691077923606</v>
+      </c>
+      <c r="AB15" s="10">
+        <v>91.98</v>
+      </c>
     </row>
     <row r="16" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C16" s="21"/>
@@ -1316,26 +1504,42 @@
       <c r="K16" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="L16" s="22"/>
-      <c r="M16" s="23"/>
+      <c r="L16" s="22">
+        <v>94.694633144244506</v>
+      </c>
+      <c r="M16" s="23">
+        <v>87.56</v>
+      </c>
       <c r="O16" s="21"/>
       <c r="P16" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="Q16" s="22"/>
-      <c r="R16" s="23"/>
+      <c r="Q16" s="22">
+        <v>96.515280236400699</v>
+      </c>
+      <c r="R16" s="23">
+        <v>87.03</v>
+      </c>
       <c r="T16" s="21"/>
       <c r="U16" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="V16" s="22"/>
-      <c r="W16" s="23"/>
+      <c r="V16" s="36">
+        <v>97.082873928417598</v>
+      </c>
+      <c r="W16" s="23">
+        <v>87.84</v>
+      </c>
       <c r="Y16" s="8"/>
       <c r="Z16" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="AA16" s="9"/>
-      <c r="AB16" s="10"/>
+      <c r="AA16" s="34">
+        <v>97.764375291161798</v>
+      </c>
+      <c r="AB16" s="10">
+        <v>86.76</v>
+      </c>
     </row>
     <row r="17" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C17" s="21" t="s">
@@ -1362,32 +1566,48 @@
       <c r="K17" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="L17" s="22"/>
-      <c r="M17" s="23"/>
+      <c r="L17" s="22">
+        <v>91.147926522397597</v>
+      </c>
+      <c r="M17" s="23">
+        <v>85.33</v>
+      </c>
       <c r="O17" s="21" t="s">
         <v>11</v>
       </c>
       <c r="P17" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="Q17" s="22"/>
-      <c r="R17" s="23"/>
+      <c r="Q17" s="22">
+        <v>94.654390676422494</v>
+      </c>
+      <c r="R17" s="23">
+        <v>85.98</v>
+      </c>
       <c r="T17" s="21" t="s">
         <v>11</v>
       </c>
       <c r="U17" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="V17" s="22"/>
-      <c r="W17" s="23"/>
+      <c r="V17" s="36">
+        <v>94.809557800717499</v>
+      </c>
+      <c r="W17" s="23">
+        <v>90.25</v>
+      </c>
       <c r="Y17" s="8" t="s">
         <v>11</v>
       </c>
       <c r="Z17" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="AA17" s="9"/>
-      <c r="AB17" s="10"/>
+      <c r="AA17" s="34">
+        <v>95.541206383771197</v>
+      </c>
+      <c r="AB17" s="10">
+        <v>90.1</v>
+      </c>
     </row>
     <row r="18" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C18" s="21"/>
@@ -1410,26 +1630,42 @@
       <c r="K18" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="L18" s="22"/>
-      <c r="M18" s="23"/>
+      <c r="L18" s="22">
+        <v>81.629911824847895</v>
+      </c>
+      <c r="M18" s="23">
+        <v>69.34</v>
+      </c>
       <c r="O18" s="21"/>
       <c r="P18" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="Q18" s="22"/>
-      <c r="R18" s="23"/>
+      <c r="Q18" s="22">
+        <v>86.487738453020896</v>
+      </c>
+      <c r="R18" s="23">
+        <v>71.72</v>
+      </c>
       <c r="T18" s="21"/>
       <c r="U18" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="V18" s="22"/>
-      <c r="W18" s="23"/>
+      <c r="V18" s="36">
+        <v>88.224547339506898</v>
+      </c>
+      <c r="W18" s="23">
+        <v>76.87</v>
+      </c>
       <c r="Y18" s="8"/>
       <c r="Z18" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="AA18" s="9"/>
-      <c r="AB18" s="10"/>
+      <c r="AA18" s="34">
+        <v>90.931657961583497</v>
+      </c>
+      <c r="AB18" s="10">
+        <v>76.88</v>
+      </c>
     </row>
     <row r="19" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C19" s="21"/>
@@ -1452,26 +1688,42 @@
       <c r="K19" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="L19" s="22"/>
-      <c r="M19" s="23"/>
+      <c r="L19" s="22">
+        <v>73.341941359279204</v>
+      </c>
+      <c r="M19" s="23">
+        <v>59.19</v>
+      </c>
       <c r="O19" s="21"/>
       <c r="P19" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="Q19" s="22"/>
-      <c r="R19" s="23"/>
+      <c r="Q19" s="22">
+        <v>75.483002967830302</v>
+      </c>
+      <c r="R19" s="23">
+        <v>59.83</v>
+      </c>
       <c r="T19" s="21"/>
       <c r="U19" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="V19" s="22"/>
-      <c r="W19" s="23"/>
+      <c r="V19" s="36">
+        <v>78.653498543930596</v>
+      </c>
+      <c r="W19" s="23">
+        <v>67.599999999999994</v>
+      </c>
       <c r="Y19" s="8"/>
       <c r="Z19" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="AA19" s="9"/>
-      <c r="AB19" s="10"/>
+      <c r="AA19" s="34">
+        <v>82.154690212955103</v>
+      </c>
+      <c r="AB19" s="10">
+        <v>67.459999999999994</v>
+      </c>
     </row>
     <row r="20" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C20" s="21"/>
@@ -1494,26 +1746,42 @@
       <c r="K20" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="L20" s="22"/>
-      <c r="M20" s="23"/>
+      <c r="L20" s="22">
+        <v>70.907524436112993</v>
+      </c>
+      <c r="M20" s="23">
+        <v>52.44</v>
+      </c>
       <c r="O20" s="21"/>
       <c r="P20" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="Q20" s="22"/>
-      <c r="R20" s="23"/>
+      <c r="Q20" s="22">
+        <v>72.685883512840306</v>
+      </c>
+      <c r="R20" s="23">
+        <v>52.57</v>
+      </c>
       <c r="T20" s="21"/>
       <c r="U20" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="V20" s="22"/>
-      <c r="W20" s="23"/>
+      <c r="V20" s="36">
+        <v>73.378405689436605</v>
+      </c>
+      <c r="W20" s="23">
+        <v>60.65</v>
+      </c>
       <c r="Y20" s="8"/>
       <c r="Z20" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="AA20" s="9"/>
-      <c r="AB20" s="10"/>
+      <c r="AA20" s="34">
+        <v>73.362430753735097</v>
+      </c>
+      <c r="AB20" s="10">
+        <v>60.65</v>
+      </c>
     </row>
     <row r="21" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C21" s="21" t="s">
@@ -1540,32 +1808,48 @@
       <c r="K21" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="L21" s="22"/>
-      <c r="M21" s="23"/>
+      <c r="L21" s="22">
+        <v>98.812157448928701</v>
+      </c>
+      <c r="M21" s="23">
+        <v>96.44</v>
+      </c>
       <c r="O21" s="21" t="s">
         <v>12</v>
       </c>
       <c r="P21" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="Q21" s="22"/>
-      <c r="R21" s="23"/>
+      <c r="Q21" s="22">
+        <v>99.257587456197697</v>
+      </c>
+      <c r="R21" s="23">
+        <v>96.59</v>
+      </c>
       <c r="T21" s="21" t="s">
         <v>12</v>
       </c>
       <c r="U21" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="V21" s="22"/>
-      <c r="W21" s="23"/>
+      <c r="V21" s="36">
+        <v>99.405747339635894</v>
+      </c>
+      <c r="W21" s="23">
+        <v>96.73</v>
+      </c>
       <c r="Y21" s="8" t="s">
         <v>12</v>
       </c>
       <c r="Z21" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="AA21" s="9"/>
-      <c r="AB21" s="10"/>
+      <c r="AA21" s="34">
+        <v>99.406080246848006</v>
+      </c>
+      <c r="AB21" s="10">
+        <v>96.73</v>
+      </c>
     </row>
     <row r="22" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C22" s="21"/>
@@ -1588,26 +1872,42 @@
       <c r="K22" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="L22" s="22"/>
-      <c r="M22" s="23"/>
+      <c r="L22" s="22">
+        <v>98.704544168208102</v>
+      </c>
+      <c r="M22" s="23">
+        <v>97.13</v>
+      </c>
       <c r="O22" s="21"/>
       <c r="P22" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="Q22" s="22"/>
-      <c r="R22" s="23"/>
+      <c r="Q22" s="22">
+        <v>99.145841399601693</v>
+      </c>
+      <c r="R22" s="23">
+        <v>98.12</v>
+      </c>
       <c r="T22" s="21"/>
       <c r="U22" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="V22" s="22"/>
-      <c r="W22" s="23"/>
+      <c r="V22" s="36">
+        <v>99.145841399601693</v>
+      </c>
+      <c r="W22" s="23">
+        <v>98.12</v>
+      </c>
       <c r="Y22" s="8"/>
       <c r="Z22" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="AA22" s="9"/>
-      <c r="AB22" s="10"/>
+      <c r="AA22" s="34">
+        <v>99.420888729189102</v>
+      </c>
+      <c r="AB22" s="10">
+        <v>98.12</v>
+      </c>
     </row>
     <row r="23" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C23" s="21"/>
@@ -1630,26 +1930,42 @@
       <c r="K23" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="L23" s="22"/>
-      <c r="M23" s="23"/>
+      <c r="L23" s="22">
+        <v>98.406471705325202</v>
+      </c>
+      <c r="M23" s="23">
+        <v>91.24</v>
+      </c>
       <c r="O23" s="21"/>
       <c r="P23" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="Q23" s="22"/>
-      <c r="R23" s="23"/>
+      <c r="Q23" s="22">
+        <v>98.837336777703896</v>
+      </c>
+      <c r="R23" s="23">
+        <v>91.06</v>
+      </c>
       <c r="T23" s="21"/>
       <c r="U23" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="V23" s="22"/>
-      <c r="W23" s="23"/>
+      <c r="V23" s="36">
+        <v>99.415675914599205</v>
+      </c>
+      <c r="W23" s="23">
+        <v>91.2</v>
+      </c>
       <c r="Y23" s="8"/>
       <c r="Z23" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="AA23" s="9"/>
-      <c r="AB23" s="10"/>
+      <c r="AA23" s="34">
+        <v>99.561389670192</v>
+      </c>
+      <c r="AB23" s="10">
+        <v>90.61</v>
+      </c>
     </row>
     <row r="24" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C24" s="24"/>
@@ -1672,26 +1988,42 @@
       <c r="K24" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="L24" s="25"/>
-      <c r="M24" s="26"/>
+      <c r="L24" s="25">
+        <v>97.562728083059596</v>
+      </c>
+      <c r="M24" s="26">
+        <v>86.58</v>
+      </c>
       <c r="O24" s="24"/>
       <c r="P24" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="Q24" s="25"/>
-      <c r="R24" s="26"/>
+      <c r="Q24" s="25">
+        <v>98.570849475026904</v>
+      </c>
+      <c r="R24" s="26">
+        <v>87.33</v>
+      </c>
       <c r="T24" s="24"/>
       <c r="U24" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="V24" s="25"/>
-      <c r="W24" s="26"/>
+      <c r="V24" s="37">
+        <v>99.284894815269993</v>
+      </c>
+      <c r="W24" s="26">
+        <v>87.6</v>
+      </c>
       <c r="Y24" s="11"/>
       <c r="Z24" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="AA24" s="12"/>
-      <c r="AB24" s="13"/>
+      <c r="AA24" s="35">
+        <v>99.429148404313693</v>
+      </c>
+      <c r="AB24" s="13">
+        <v>86.73</v>
+      </c>
     </row>
     <row r="27" spans="3:28" x14ac:dyDescent="0.2">
       <c r="J27" s="1" t="s">
@@ -1776,24 +2108,36 @@
       <c r="K29" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="L29" s="9"/>
-      <c r="M29" s="10"/>
+      <c r="L29" s="34">
+        <v>99.291809243086405</v>
+      </c>
+      <c r="M29" s="10">
+        <v>98.29</v>
+      </c>
       <c r="O29" s="8" t="s">
         <v>0</v>
       </c>
       <c r="P29" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="Q29" s="9"/>
-      <c r="R29" s="10"/>
+      <c r="Q29" s="34">
+        <v>99.286751324742198</v>
+      </c>
+      <c r="R29" s="10">
+        <v>98.43</v>
+      </c>
       <c r="T29" s="8" t="s">
         <v>0</v>
       </c>
       <c r="U29" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="V29" s="9"/>
-      <c r="W29" s="10"/>
+      <c r="V29" s="34">
+        <v>99.437427660605707</v>
+      </c>
+      <c r="W29" s="10">
+        <v>98.86</v>
+      </c>
       <c r="Y29" s="8" t="s">
         <v>0</v>
       </c>
@@ -1803,27 +2147,41 @@
       <c r="AA29" s="9">
         <v>99.3</v>
       </c>
-      <c r="AB29" s="10"/>
+      <c r="AB29" s="10">
+        <v>98.86</v>
+      </c>
     </row>
     <row r="30" spans="3:28" x14ac:dyDescent="0.2">
       <c r="J30" s="8"/>
       <c r="K30" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="L30" s="9"/>
-      <c r="M30" s="10"/>
+      <c r="L30" s="34">
+        <v>99.718430602154697</v>
+      </c>
+      <c r="M30" s="10">
+        <v>97.42</v>
+      </c>
       <c r="O30" s="8"/>
       <c r="P30" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="Q30" s="9"/>
-      <c r="R30" s="10"/>
+      <c r="Q30" s="34">
+        <v>99.727306186636298</v>
+      </c>
+      <c r="R30" s="10">
+        <v>97.45</v>
+      </c>
       <c r="T30" s="8"/>
       <c r="U30" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="V30" s="9"/>
-      <c r="W30" s="10"/>
+      <c r="V30" s="34">
+        <v>99.863658225465798</v>
+      </c>
+      <c r="W30" s="10">
+        <v>98.73</v>
+      </c>
       <c r="Y30" s="8"/>
       <c r="Z30" s="9" t="s">
         <v>2</v>
@@ -1831,27 +2189,41 @@
       <c r="AA30" s="9">
         <v>99.86</v>
       </c>
-      <c r="AB30" s="10"/>
+      <c r="AB30" s="10">
+        <v>98.73</v>
+      </c>
     </row>
     <row r="31" spans="3:28" x14ac:dyDescent="0.2">
       <c r="J31" s="8"/>
       <c r="K31" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="L31" s="9"/>
-      <c r="M31" s="10"/>
+      <c r="L31" s="34">
+        <v>99.557056500397493</v>
+      </c>
+      <c r="M31" s="10">
+        <v>96.73</v>
+      </c>
       <c r="O31" s="8"/>
       <c r="P31" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="Q31" s="9"/>
-      <c r="R31" s="10"/>
+      <c r="Q31" s="34">
+        <v>99.557485453805995</v>
+      </c>
+      <c r="R31" s="10">
+        <v>96.6</v>
+      </c>
       <c r="T31" s="8"/>
       <c r="U31" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="V31" s="9"/>
-      <c r="W31" s="10"/>
+      <c r="V31" s="34">
+        <v>99.562562667966205</v>
+      </c>
+      <c r="W31" s="10">
+        <v>98.85</v>
+      </c>
       <c r="Y31" s="8"/>
       <c r="Z31" s="9" t="s">
         <v>3</v>
@@ -1859,27 +2231,41 @@
       <c r="AA31" s="9">
         <v>99.56</v>
       </c>
-      <c r="AB31" s="10"/>
+      <c r="AB31" s="10">
+        <v>98.85</v>
+      </c>
     </row>
     <row r="32" spans="3:28" x14ac:dyDescent="0.2">
       <c r="J32" s="8"/>
       <c r="K32" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="L32" s="9"/>
-      <c r="M32" s="10"/>
+      <c r="L32" s="34">
+        <v>99.278134262279593</v>
+      </c>
+      <c r="M32" s="10">
+        <v>96.41</v>
+      </c>
       <c r="O32" s="8"/>
       <c r="P32" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="Q32" s="9"/>
-      <c r="R32" s="10"/>
+      <c r="Q32" s="34">
+        <v>99.419274106080806</v>
+      </c>
+      <c r="R32" s="10">
+        <v>94.04</v>
+      </c>
       <c r="T32" s="8"/>
       <c r="U32" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="V32" s="9"/>
-      <c r="W32" s="10"/>
+      <c r="V32" s="34">
+        <v>99.435311533732104</v>
+      </c>
+      <c r="W32" s="10">
+        <v>97.29</v>
+      </c>
       <c r="Y32" s="8"/>
       <c r="Z32" s="9" t="s">
         <v>4</v>
@@ -1887,27 +2273,41 @@
       <c r="AA32" s="9">
         <v>99.57</v>
       </c>
-      <c r="AB32" s="10"/>
+      <c r="AB32" s="10">
+        <v>97.29</v>
+      </c>
     </row>
     <row r="33" spans="10:28" x14ac:dyDescent="0.2">
       <c r="J33" s="8"/>
       <c r="K33" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="L33" s="9"/>
-      <c r="M33" s="10"/>
+      <c r="L33" s="34">
+        <v>99.695824357606298</v>
+      </c>
+      <c r="M33" s="10">
+        <v>97.27</v>
+      </c>
       <c r="O33" s="8"/>
       <c r="P33" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="Q33" s="9"/>
-      <c r="R33" s="10"/>
+      <c r="Q33" s="34">
+        <v>99.695824357606298</v>
+      </c>
+      <c r="R33" s="10">
+        <v>91.52</v>
+      </c>
       <c r="T33" s="8"/>
       <c r="U33" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="V33" s="9"/>
-      <c r="W33" s="10"/>
+      <c r="V33" s="34">
+        <v>99.5456400230876</v>
+      </c>
+      <c r="W33" s="10">
+        <v>95.47</v>
+      </c>
       <c r="Y33" s="8"/>
       <c r="Z33" s="9" t="s">
         <v>5</v>
@@ -1915,27 +2315,41 @@
       <c r="AA33" s="9">
         <v>99.7</v>
       </c>
-      <c r="AB33" s="10"/>
+      <c r="AB33" s="10">
+        <v>95.47</v>
+      </c>
     </row>
     <row r="34" spans="10:28" x14ac:dyDescent="0.2">
       <c r="J34" s="8"/>
       <c r="K34" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="L34" s="9"/>
-      <c r="M34" s="10"/>
+      <c r="L34" s="34">
+        <v>99.419140829703693</v>
+      </c>
+      <c r="M34" s="10">
+        <v>94.81</v>
+      </c>
       <c r="O34" s="8"/>
       <c r="P34" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="Q34" s="9"/>
-      <c r="R34" s="10"/>
+      <c r="Q34" s="34">
+        <v>99.562345704744303</v>
+      </c>
+      <c r="R34" s="10">
+        <v>86.6</v>
+      </c>
       <c r="T34" s="8"/>
       <c r="U34" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="V34" s="9"/>
-      <c r="W34" s="10"/>
+      <c r="V34" s="34">
+        <v>99.562345704744303</v>
+      </c>
+      <c r="W34" s="10">
+        <v>86.6</v>
+      </c>
       <c r="Y34" s="8"/>
       <c r="Z34" s="9" t="s">
         <v>6</v>
@@ -1943,27 +2357,41 @@
       <c r="AA34" s="9">
         <v>99.71</v>
       </c>
-      <c r="AB34" s="10"/>
+      <c r="AB34" s="10">
+        <v>87.06</v>
+      </c>
     </row>
     <row r="35" spans="10:28" x14ac:dyDescent="0.2">
       <c r="J35" s="8"/>
       <c r="K35" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="L35" s="9"/>
-      <c r="M35" s="10"/>
+      <c r="L35" s="34">
+        <v>99.016179267225297</v>
+      </c>
+      <c r="M35" s="10">
+        <v>93.4</v>
+      </c>
       <c r="O35" s="8"/>
       <c r="P35" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="Q35" s="9"/>
-      <c r="R35" s="10"/>
+      <c r="Q35" s="34">
+        <v>99.154784846329704</v>
+      </c>
+      <c r="R35" s="10">
+        <v>82.61</v>
+      </c>
       <c r="T35" s="8"/>
       <c r="U35" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="V35" s="9"/>
-      <c r="W35" s="10"/>
+      <c r="V35" s="34">
+        <v>99.297085790328296</v>
+      </c>
+      <c r="W35" s="10">
+        <v>82.47</v>
+      </c>
       <c r="Y35" s="8"/>
       <c r="Z35" s="9" t="s">
         <v>7</v>
@@ -1971,27 +2399,41 @@
       <c r="AA35" s="9">
         <v>99.3</v>
       </c>
-      <c r="AB35" s="10"/>
+      <c r="AB35" s="10">
+        <v>82.46</v>
+      </c>
     </row>
     <row r="36" spans="10:28" x14ac:dyDescent="0.2">
       <c r="J36" s="8"/>
       <c r="K36" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="L36" s="9"/>
-      <c r="M36" s="10"/>
+      <c r="L36" s="34">
+        <v>98.844172789062895</v>
+      </c>
+      <c r="M36" s="10">
+        <v>90.02</v>
+      </c>
       <c r="O36" s="8"/>
       <c r="P36" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="Q36" s="9"/>
-      <c r="R36" s="10"/>
+      <c r="Q36" s="34">
+        <v>98.8442690766353</v>
+      </c>
+      <c r="R36" s="10">
+        <v>76.38</v>
+      </c>
       <c r="T36" s="8"/>
       <c r="U36" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="V36" s="9"/>
-      <c r="W36" s="10"/>
+      <c r="V36" s="34">
+        <v>98.988531710822997</v>
+      </c>
+      <c r="W36" s="10">
+        <v>78.930000000000007</v>
+      </c>
       <c r="Y36" s="8"/>
       <c r="Z36" s="9" t="s">
         <v>8</v>
@@ -1999,7 +2441,9 @@
       <c r="AA36" s="9">
         <v>99.13</v>
       </c>
-      <c r="AB36" s="10"/>
+      <c r="AB36" s="10">
+        <v>79.22</v>
+      </c>
     </row>
     <row r="37" spans="10:28" x14ac:dyDescent="0.2">
       <c r="J37" s="8" t="s">
@@ -2008,24 +2452,36 @@
       <c r="K37" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="L37" s="9"/>
-      <c r="M37" s="10"/>
+      <c r="L37" s="34">
+        <v>98.832260982766698</v>
+      </c>
+      <c r="M37" s="10">
+        <v>97.35</v>
+      </c>
       <c r="O37" s="8" t="s">
         <v>9</v>
       </c>
       <c r="P37" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="Q37" s="9"/>
-      <c r="R37" s="10"/>
+      <c r="Q37" s="34">
+        <v>99.412022746388999</v>
+      </c>
+      <c r="R37" s="10">
+        <v>97.35</v>
+      </c>
       <c r="T37" s="8" t="s">
         <v>9</v>
       </c>
       <c r="U37" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="V37" s="9"/>
-      <c r="W37" s="10"/>
+      <c r="V37" s="34">
+        <v>99.559884559884594</v>
+      </c>
+      <c r="W37" s="10">
+        <v>97.49</v>
+      </c>
       <c r="Y37" s="8" t="s">
         <v>9</v>
       </c>
@@ -2035,27 +2491,41 @@
       <c r="AA37" s="9">
         <v>99.56</v>
       </c>
-      <c r="AB37" s="10"/>
+      <c r="AB37" s="10">
+        <v>97.49</v>
+      </c>
     </row>
     <row r="38" spans="10:28" x14ac:dyDescent="0.2">
       <c r="J38" s="8"/>
       <c r="K38" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="L38" s="9"/>
-      <c r="M38" s="10"/>
+      <c r="L38" s="34">
+        <v>99.321683383310898</v>
+      </c>
+      <c r="M38" s="10">
+        <v>93.47</v>
+      </c>
       <c r="O38" s="8"/>
       <c r="P38" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="Q38" s="9"/>
-      <c r="R38" s="10"/>
+      <c r="Q38" s="34">
+        <v>99.444209125115506</v>
+      </c>
+      <c r="R38" s="10">
+        <v>93.23</v>
+      </c>
       <c r="T38" s="8"/>
       <c r="U38" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="V38" s="9"/>
-      <c r="W38" s="10"/>
+      <c r="V38" s="34">
+        <v>99.714977597725394</v>
+      </c>
+      <c r="W38" s="10">
+        <v>94.96</v>
+      </c>
       <c r="Y38" s="8"/>
       <c r="Z38" s="9" t="s">
         <v>2</v>
@@ -2063,7 +2533,9 @@
       <c r="AA38" s="9">
         <v>99.71</v>
       </c>
-      <c r="AB38" s="10"/>
+      <c r="AB38" s="10">
+        <v>94.96</v>
+      </c>
     </row>
     <row r="39" spans="10:28" x14ac:dyDescent="0.2">
       <c r="J39" s="8" t="s">
@@ -2072,24 +2544,36 @@
       <c r="K39" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="L39" s="9"/>
-      <c r="M39" s="10"/>
+      <c r="L39" s="34">
+        <v>98.6943123585839</v>
+      </c>
+      <c r="M39" s="10">
+        <v>92.12</v>
+      </c>
       <c r="O39" s="8" t="s">
         <v>10</v>
       </c>
       <c r="P39" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="Q39" s="9"/>
-      <c r="R39" s="10"/>
+      <c r="Q39" s="34">
+        <v>98.991989399144998</v>
+      </c>
+      <c r="R39" s="10">
+        <v>85.68</v>
+      </c>
       <c r="T39" s="8" t="s">
         <v>10</v>
       </c>
       <c r="U39" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="V39" s="9"/>
-      <c r="W39" s="10"/>
+      <c r="V39" s="34">
+        <v>99.415003006576299</v>
+      </c>
+      <c r="W39" s="10">
+        <v>86.22</v>
+      </c>
       <c r="Y39" s="8" t="s">
         <v>10</v>
       </c>
@@ -2099,27 +2583,41 @@
       <c r="AA39" s="9">
         <v>99.43</v>
       </c>
-      <c r="AB39" s="10"/>
+      <c r="AB39" s="10">
+        <v>86.22</v>
+      </c>
     </row>
     <row r="40" spans="10:28" x14ac:dyDescent="0.2">
       <c r="J40" s="8"/>
       <c r="K40" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="L40" s="9"/>
-      <c r="M40" s="10"/>
+      <c r="L40" s="34">
+        <v>98.460603284465705</v>
+      </c>
+      <c r="M40" s="10">
+        <v>86.76</v>
+      </c>
       <c r="O40" s="8"/>
       <c r="P40" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="Q40" s="9"/>
-      <c r="R40" s="10"/>
+      <c r="Q40" s="34">
+        <v>99.015448244999703</v>
+      </c>
+      <c r="R40" s="10">
+        <v>78.540000000000006</v>
+      </c>
       <c r="T40" s="8"/>
       <c r="U40" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="V40" s="9"/>
-      <c r="W40" s="10"/>
+      <c r="V40" s="34">
+        <v>99.165946413137405</v>
+      </c>
+      <c r="W40" s="10">
+        <v>79.87</v>
+      </c>
       <c r="Y40" s="8"/>
       <c r="Z40" s="9" t="s">
         <v>4</v>
@@ -2127,7 +2625,9 @@
       <c r="AA40" s="9">
         <v>99.3</v>
       </c>
-      <c r="AB40" s="10"/>
+      <c r="AB40" s="10">
+        <v>80.28</v>
+      </c>
     </row>
     <row r="41" spans="10:28" x14ac:dyDescent="0.2">
       <c r="J41" s="8" t="s">
@@ -2136,24 +2636,36 @@
       <c r="K41" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="L41" s="9"/>
-      <c r="M41" s="10"/>
+      <c r="L41" s="34">
+        <v>96.1293845221943</v>
+      </c>
+      <c r="M41" s="10">
+        <v>90.4</v>
+      </c>
       <c r="O41" s="8" t="s">
         <v>11</v>
       </c>
       <c r="P41" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="Q41" s="9"/>
-      <c r="R41" s="10"/>
+      <c r="Q41" s="34">
+        <v>96.582893546840396</v>
+      </c>
+      <c r="R41" s="10">
+        <v>90.84</v>
+      </c>
       <c r="T41" s="8" t="s">
         <v>11</v>
       </c>
       <c r="U41" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="V41" s="9"/>
-      <c r="W41" s="10"/>
+      <c r="V41" s="34">
+        <v>96.582893546840396</v>
+      </c>
+      <c r="W41" s="10">
+        <v>92.01</v>
+      </c>
       <c r="Y41" s="8" t="s">
         <v>11</v>
       </c>
@@ -2163,27 +2675,41 @@
       <c r="AA41" s="9">
         <v>96.44</v>
       </c>
-      <c r="AB41" s="10"/>
+      <c r="AB41" s="10">
+        <v>92.01</v>
+      </c>
     </row>
     <row r="42" spans="10:28" x14ac:dyDescent="0.2">
       <c r="J42" s="8"/>
       <c r="K42" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="L42" s="9"/>
-      <c r="M42" s="10"/>
+      <c r="L42" s="34">
+        <v>91.423141791576597</v>
+      </c>
+      <c r="M42" s="10">
+        <v>78.02</v>
+      </c>
       <c r="O42" s="8"/>
       <c r="P42" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="Q42" s="9"/>
-      <c r="R42" s="10"/>
+      <c r="Q42" s="34">
+        <v>93.302766388734199</v>
+      </c>
+      <c r="R42" s="10">
+        <v>78.67</v>
+      </c>
       <c r="T42" s="8"/>
       <c r="U42" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="V42" s="9"/>
-      <c r="W42" s="10"/>
+      <c r="V42" s="34">
+        <v>93.442317389910599</v>
+      </c>
+      <c r="W42" s="10">
+        <v>78.67</v>
+      </c>
       <c r="Y42" s="8"/>
       <c r="Z42" s="9" t="s">
         <v>2</v>
@@ -2191,27 +2717,41 @@
       <c r="AA42" s="9">
         <v>93.44</v>
       </c>
-      <c r="AB42" s="10"/>
+      <c r="AB42" s="10">
+        <v>79.94</v>
+      </c>
     </row>
     <row r="43" spans="10:28" x14ac:dyDescent="0.2">
       <c r="J43" s="8"/>
       <c r="K43" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="L43" s="9"/>
-      <c r="M43" s="10"/>
+      <c r="L43" s="34">
+        <v>82.728818217052606</v>
+      </c>
+      <c r="M43" s="10">
+        <v>67.47</v>
+      </c>
       <c r="O43" s="8"/>
       <c r="P43" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="Q43" s="9"/>
-      <c r="R43" s="10"/>
+      <c r="Q43" s="34">
+        <v>82.880996223891501</v>
+      </c>
+      <c r="R43" s="10">
+        <v>67.75</v>
+      </c>
       <c r="T43" s="8"/>
       <c r="U43" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="V43" s="9"/>
-      <c r="W43" s="10"/>
+      <c r="V43" s="34">
+        <v>82.052981256516603</v>
+      </c>
+      <c r="W43" s="10">
+        <v>67.89</v>
+      </c>
       <c r="Y43" s="8"/>
       <c r="Z43" s="9" t="s">
         <v>3</v>
@@ -2219,27 +2759,41 @@
       <c r="AA43" s="9">
         <v>82.34</v>
       </c>
-      <c r="AB43" s="10"/>
+      <c r="AB43" s="10">
+        <v>68.319999999999993</v>
+      </c>
     </row>
     <row r="44" spans="10:28" x14ac:dyDescent="0.2">
       <c r="J44" s="8"/>
       <c r="K44" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="L44" s="9"/>
-      <c r="M44" s="10"/>
+      <c r="L44" s="34">
+        <v>73.576345245828605</v>
+      </c>
+      <c r="M44" s="10">
+        <v>60.65</v>
+      </c>
       <c r="O44" s="8"/>
       <c r="P44" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="Q44" s="9"/>
-      <c r="R44" s="10"/>
+      <c r="Q44" s="34">
+        <v>73.234084342379603</v>
+      </c>
+      <c r="R44" s="10">
+        <v>60.97</v>
+      </c>
       <c r="T44" s="8"/>
       <c r="U44" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="V44" s="9"/>
-      <c r="W44" s="10"/>
+      <c r="V44" s="34">
+        <v>73.654970760233894</v>
+      </c>
+      <c r="W44" s="10">
+        <v>60.97</v>
+      </c>
       <c r="Y44" s="8"/>
       <c r="Z44" s="9" t="s">
         <v>4</v>
@@ -2247,7 +2801,9 @@
       <c r="AA44" s="9">
         <v>70.75</v>
       </c>
-      <c r="AB44" s="10"/>
+      <c r="AB44" s="10">
+        <v>61.32</v>
+      </c>
     </row>
     <row r="45" spans="10:28" x14ac:dyDescent="0.2">
       <c r="J45" s="8" t="s">
@@ -2256,24 +2812,36 @@
       <c r="K45" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="L45" s="9"/>
-      <c r="M45" s="10"/>
+      <c r="L45" s="34">
+        <v>99.554222512587998</v>
+      </c>
+      <c r="M45" s="10">
+        <v>96.73</v>
+      </c>
       <c r="O45" s="8" t="s">
         <v>12</v>
       </c>
       <c r="P45" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="Q45" s="9"/>
-      <c r="R45" s="10"/>
+      <c r="Q45" s="34">
+        <v>99.554222512587998</v>
+      </c>
+      <c r="R45" s="10">
+        <v>96.73</v>
+      </c>
       <c r="T45" s="8" t="s">
         <v>12</v>
       </c>
       <c r="U45" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="V45" s="9"/>
-      <c r="W45" s="10"/>
+      <c r="V45" s="34">
+        <v>99.554222512587998</v>
+      </c>
+      <c r="W45" s="10">
+        <v>96.73</v>
+      </c>
       <c r="Y45" s="8" t="s">
         <v>12</v>
       </c>
@@ -2283,27 +2851,41 @@
       <c r="AA45" s="9">
         <v>99.55</v>
       </c>
-      <c r="AB45" s="10"/>
+      <c r="AB45" s="10">
+        <v>96.43</v>
+      </c>
     </row>
     <row r="46" spans="10:28" x14ac:dyDescent="0.2">
       <c r="J46" s="8"/>
       <c r="K46" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="L46" s="9"/>
-      <c r="M46" s="10"/>
+      <c r="L46" s="34">
+        <v>99.572447336422499</v>
+      </c>
+      <c r="M46" s="10">
+        <v>98.12</v>
+      </c>
       <c r="O46" s="8"/>
       <c r="P46" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="Q46" s="9"/>
-      <c r="R46" s="10"/>
+      <c r="Q46" s="34">
+        <v>99.717387269254502</v>
+      </c>
+      <c r="R46" s="10">
+        <v>98.12</v>
+      </c>
       <c r="T46" s="8"/>
       <c r="U46" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="V46" s="9"/>
-      <c r="W46" s="10"/>
+      <c r="V46" s="34">
+        <v>99.858680307609802</v>
+      </c>
+      <c r="W46" s="10">
+        <v>98.12</v>
+      </c>
       <c r="Y46" s="8"/>
       <c r="Z46" s="9" t="s">
         <v>2</v>
@@ -2311,27 +2893,41 @@
       <c r="AA46" s="9">
         <v>99.86</v>
       </c>
-      <c r="AB46" s="10"/>
+      <c r="AB46" s="10">
+        <v>98.12</v>
+      </c>
     </row>
     <row r="47" spans="10:28" x14ac:dyDescent="0.2">
       <c r="J47" s="8"/>
       <c r="K47" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="L47" s="9"/>
-      <c r="M47" s="10"/>
+      <c r="L47" s="34">
+        <v>99.561389670192</v>
+      </c>
+      <c r="M47" s="10">
+        <v>90.61</v>
+      </c>
       <c r="O47" s="8"/>
       <c r="P47" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="Q47" s="9"/>
-      <c r="R47" s="10"/>
+      <c r="Q47" s="34">
+        <v>99.561389670192</v>
+      </c>
+      <c r="R47" s="10">
+        <v>80.239999999999995</v>
+      </c>
       <c r="T47" s="8"/>
       <c r="U47" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="V47" s="9"/>
-      <c r="W47" s="10"/>
+      <c r="V47" s="34">
+        <v>99.561389670192</v>
+      </c>
+      <c r="W47" s="10">
+        <v>89.42</v>
+      </c>
       <c r="Y47" s="8"/>
       <c r="Z47" s="9" t="s">
         <v>3</v>
@@ -2339,27 +2935,41 @@
       <c r="AA47" s="9">
         <v>99.56</v>
       </c>
-      <c r="AB47" s="10"/>
+      <c r="AB47" s="10">
+        <v>89.86</v>
+      </c>
     </row>
     <row r="48" spans="10:28" x14ac:dyDescent="0.2">
       <c r="J48" s="11"/>
       <c r="K48" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="L48" s="12"/>
-      <c r="M48" s="13"/>
+      <c r="L48" s="35">
+        <v>99.719868173258007</v>
+      </c>
+      <c r="M48" s="13">
+        <v>86.44</v>
+      </c>
       <c r="O48" s="11"/>
       <c r="P48" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="Q48" s="12"/>
-      <c r="R48" s="13"/>
+      <c r="Q48" s="35">
+        <v>99.719868173258007</v>
+      </c>
+      <c r="R48" s="13">
+        <v>69.02</v>
+      </c>
       <c r="T48" s="11"/>
       <c r="U48" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="V48" s="12"/>
-      <c r="W48" s="13"/>
+      <c r="V48" s="35">
+        <v>99.719868173258007</v>
+      </c>
+      <c r="W48" s="13">
+        <v>69.62</v>
+      </c>
       <c r="Y48" s="11"/>
       <c r="Z48" s="12" t="s">
         <v>4</v>
@@ -2367,7 +2977,9 @@
       <c r="AA48" s="12">
         <v>99.72</v>
       </c>
-      <c r="AB48" s="13"/>
+      <c r="AB48" s="13">
+        <v>70.209999999999994</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Finished investigating normalization, Manhattan, and window shifting
</commit_message>
<xml_diff>
--- a/results/validate_results.xlsx
+++ b/results/validate_results.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emily/Library/CloudStorage/GoogleDrive-u0835353@gcloud.utah.edu/.shortcut-targets-by-id/109kT4myKnMujFK8ni-DWM3IQ1FnMmvXr/EYANG/BCI Project/FWHT_FeatureExtract/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71ED00B3-3AA7-BE44-AAE3-CB2B52D1902B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A92D5BD-335D-864E-AF1A-DFF409ED678C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-22140" yWindow="-21120" windowWidth="38400" windowHeight="21120" xr2:uid="{AFAE147A-AF5E-4547-B045-936377B9E7D9}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16240" xr2:uid="{AFAE147A-AF5E-4547-B045-936377B9E7D9}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sliding Window" sheetId="1" r:id="rId1"/>
+    <sheet name="baseline_slidingWindow" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -316,21 +316,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
@@ -339,34 +339,33 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -758,14 +757,14 @@
       <c r="D4" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="E4" s="27" t="s">
+      <c r="E4" s="35" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="27"/>
-      <c r="G4" s="27" t="s">
+      <c r="F4" s="35"/>
+      <c r="G4" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="H4" s="28"/>
+      <c r="H4" s="36"/>
       <c r="J4" s="17" t="s">
         <v>33</v>
       </c>
@@ -819,55 +818,55 @@
       <c r="C5" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="E5" s="22">
+      <c r="D5" t="s">
+        <v>1</v>
+      </c>
+      <c r="E5">
         <v>97.88</v>
       </c>
-      <c r="F5" s="22" t="s">
+      <c r="F5" t="s">
         <v>19</v>
       </c>
-      <c r="G5" s="22">
+      <c r="G5">
         <v>96.15</v>
       </c>
-      <c r="H5" s="23" t="s">
+      <c r="H5" s="22" t="s">
         <v>26</v>
       </c>
       <c r="J5" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="K5" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="L5" s="22">
+      <c r="K5" t="s">
+        <v>1</v>
+      </c>
+      <c r="L5">
         <v>98.574854454457494</v>
       </c>
-      <c r="M5" s="23">
+      <c r="M5" s="22">
         <v>97.43</v>
       </c>
       <c r="O5" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="P5" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="Q5" s="22">
+      <c r="P5" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q5">
         <v>99.002890240902701</v>
       </c>
-      <c r="R5" s="23">
+      <c r="R5" s="22">
         <v>97.57</v>
       </c>
       <c r="T5" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="U5" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="V5" s="36">
+      <c r="U5" t="s">
+        <v>1</v>
+      </c>
+      <c r="V5" s="33">
         <v>99.002890240902701</v>
       </c>
-      <c r="W5" s="23">
+      <c r="W5" s="22">
         <v>97.86</v>
       </c>
       <c r="Y5" s="8" t="s">
@@ -876,7 +875,7 @@
       <c r="Z5" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="AA5" s="34">
+      <c r="AA5" s="31">
         <v>99.148302585035395</v>
       </c>
       <c r="AB5" s="10">
@@ -885,56 +884,56 @@
     </row>
     <row r="6" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C6" s="21"/>
-      <c r="D6" s="22" t="s">
-        <v>2</v>
-      </c>
-      <c r="E6" s="22">
+      <c r="D6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E6">
         <v>97.56</v>
       </c>
-      <c r="F6" s="22" t="s">
+      <c r="F6" t="s">
         <v>25</v>
       </c>
-      <c r="G6" s="22">
+      <c r="G6">
         <v>96.08</v>
       </c>
-      <c r="H6" s="23" t="s">
+      <c r="H6" s="22" t="s">
         <v>26</v>
       </c>
       <c r="J6" s="21"/>
-      <c r="K6" s="22" t="s">
-        <v>2</v>
-      </c>
-      <c r="L6" s="22">
+      <c r="K6" t="s">
+        <v>2</v>
+      </c>
+      <c r="L6">
         <v>98.577017107872706</v>
       </c>
-      <c r="M6" s="23">
+      <c r="M6" s="22">
         <v>96.76</v>
       </c>
       <c r="O6" s="21"/>
-      <c r="P6" s="22" t="s">
-        <v>2</v>
-      </c>
-      <c r="Q6" s="22">
+      <c r="P6" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q6">
         <v>98.687480598085301</v>
       </c>
-      <c r="R6" s="23">
+      <c r="R6" s="22">
         <v>97.04</v>
       </c>
       <c r="T6" s="21"/>
-      <c r="U6" s="22" t="s">
-        <v>2</v>
-      </c>
-      <c r="V6" s="36">
+      <c r="U6" t="s">
+        <v>2</v>
+      </c>
+      <c r="V6" s="33">
         <v>99.563480747068098</v>
       </c>
-      <c r="W6" s="23">
+      <c r="W6" s="22">
         <v>97.04</v>
       </c>
       <c r="Y6" s="8"/>
       <c r="Z6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="AA6" s="34">
+      <c r="AA6" s="31">
         <v>99.454557622808196</v>
       </c>
       <c r="AB6" s="10">
@@ -943,56 +942,56 @@
     </row>
     <row r="7" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C7" s="21"/>
-      <c r="D7" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="E7" s="22">
+      <c r="D7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E7">
         <v>97.49</v>
       </c>
-      <c r="F7" s="22" t="s">
+      <c r="F7" t="s">
         <v>24</v>
       </c>
-      <c r="G7" s="22">
+      <c r="G7">
         <v>97.06</v>
       </c>
-      <c r="H7" s="23" t="s">
+      <c r="H7" s="22" t="s">
         <v>26</v>
       </c>
       <c r="J7" s="21"/>
-      <c r="K7" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="L7" s="22">
+      <c r="K7" t="s">
+        <v>3</v>
+      </c>
+      <c r="L7">
         <v>98.6800879070761</v>
       </c>
-      <c r="M7" s="23">
+      <c r="M7" s="22">
         <v>97.06</v>
       </c>
       <c r="O7" s="21"/>
-      <c r="P7" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q7" s="22">
+      <c r="P7" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q7">
         <v>99.263354797323302</v>
       </c>
-      <c r="R7" s="23">
+      <c r="R7" s="22">
         <v>96.73</v>
       </c>
       <c r="T7" s="21"/>
-      <c r="U7" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="V7" s="36">
+      <c r="U7" t="s">
+        <v>3</v>
+      </c>
+      <c r="V7" s="33">
         <v>99.263354797323302</v>
       </c>
-      <c r="W7" s="23">
+      <c r="W7" s="22">
         <v>96.73</v>
       </c>
       <c r="Y7" s="8"/>
       <c r="Z7" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="AA7" s="34">
+      <c r="AA7" s="31">
         <v>99.413444199559194</v>
       </c>
       <c r="AB7" s="10">
@@ -1001,56 +1000,56 @@
     </row>
     <row r="8" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C8" s="21"/>
-      <c r="D8" s="22" t="s">
-        <v>4</v>
-      </c>
-      <c r="E8" s="22">
+      <c r="D8" t="s">
+        <v>4</v>
+      </c>
+      <c r="E8">
         <v>96.11</v>
       </c>
-      <c r="F8" s="22" t="s">
+      <c r="F8" t="s">
         <v>23</v>
       </c>
-      <c r="G8" s="22">
+      <c r="G8">
         <v>94.68</v>
       </c>
-      <c r="H8" s="23" t="s">
+      <c r="H8" s="22" t="s">
         <v>26</v>
       </c>
       <c r="J8" s="21"/>
-      <c r="K8" s="22" t="s">
-        <v>4</v>
-      </c>
-      <c r="L8" s="22">
+      <c r="K8" t="s">
+        <v>4</v>
+      </c>
+      <c r="L8">
         <v>97.531177473946698</v>
       </c>
-      <c r="M8" s="23">
+      <c r="M8" s="22">
         <v>95.52</v>
       </c>
       <c r="O8" s="21"/>
-      <c r="P8" s="22" t="s">
-        <v>4</v>
-      </c>
-      <c r="Q8" s="22">
+      <c r="P8" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q8">
         <v>97.985950453055693</v>
       </c>
-      <c r="R8" s="23">
+      <c r="R8" s="22">
         <v>96.54</v>
       </c>
       <c r="T8" s="21"/>
-      <c r="U8" s="22" t="s">
-        <v>4</v>
-      </c>
-      <c r="V8" s="36">
+      <c r="U8" t="s">
+        <v>4</v>
+      </c>
+      <c r="V8" s="33">
         <v>98.986707472223003</v>
       </c>
-      <c r="W8" s="23">
+      <c r="W8" s="22">
         <v>96.54</v>
       </c>
       <c r="Y8" s="8"/>
       <c r="Z8" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="AA8" s="34">
+      <c r="AA8" s="31">
         <v>98.856727876335697</v>
       </c>
       <c r="AB8" s="10">
@@ -1059,56 +1058,56 @@
     </row>
     <row r="9" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C9" s="21"/>
-      <c r="D9" s="22" t="s">
+      <c r="D9" t="s">
         <v>5</v>
       </c>
-      <c r="E9" s="22">
+      <c r="E9">
         <v>97.56</v>
       </c>
-      <c r="F9" s="22" t="s">
+      <c r="F9" t="s">
         <v>21</v>
       </c>
-      <c r="G9" s="22">
+      <c r="G9">
         <v>96.21</v>
       </c>
-      <c r="H9" s="23" t="s">
+      <c r="H9" s="22" t="s">
         <v>27</v>
       </c>
       <c r="J9" s="21"/>
-      <c r="K9" s="22" t="s">
+      <c r="K9" t="s">
         <v>5</v>
       </c>
-      <c r="L9" s="22">
+      <c r="L9">
         <v>98.633530623712701</v>
       </c>
-      <c r="M9" s="23">
+      <c r="M9" s="22">
         <v>97.11</v>
       </c>
       <c r="O9" s="21"/>
-      <c r="P9" s="22" t="s">
+      <c r="P9" t="s">
         <v>5</v>
       </c>
-      <c r="Q9" s="22">
+      <c r="Q9">
         <v>99.086401427689395</v>
       </c>
-      <c r="R9" s="23">
+      <c r="R9" s="22">
         <v>97.42</v>
       </c>
       <c r="T9" s="21"/>
-      <c r="U9" s="22" t="s">
+      <c r="U9" t="s">
         <v>5</v>
       </c>
-      <c r="V9" s="36">
+      <c r="V9" s="33">
         <v>99.395047491992898</v>
       </c>
-      <c r="W9" s="23">
+      <c r="W9" s="22">
         <v>97.42</v>
       </c>
       <c r="Y9" s="8"/>
       <c r="Z9" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="AA9" s="34">
+      <c r="AA9" s="31">
         <v>99.695824357606298</v>
       </c>
       <c r="AB9" s="10">
@@ -1117,56 +1116,56 @@
     </row>
     <row r="10" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C10" s="21"/>
-      <c r="D10" s="22" t="s">
+      <c r="D10" t="s">
         <v>6</v>
       </c>
-      <c r="E10" s="22">
+      <c r="E10">
         <v>96.38</v>
       </c>
-      <c r="F10" s="22" t="s">
+      <c r="F10" t="s">
         <v>21</v>
       </c>
-      <c r="G10" s="22">
+      <c r="G10">
         <v>93.66</v>
       </c>
-      <c r="H10" s="23" t="s">
+      <c r="H10" s="22" t="s">
         <v>27</v>
       </c>
       <c r="J10" s="21"/>
-      <c r="K10" s="22" t="s">
+      <c r="K10" t="s">
         <v>6</v>
       </c>
-      <c r="L10" s="22">
+      <c r="L10">
         <v>97.541939235450499</v>
       </c>
-      <c r="M10" s="23">
+      <c r="M10" s="22">
         <v>94.81</v>
       </c>
       <c r="O10" s="21"/>
-      <c r="P10" s="22" t="s">
+      <c r="P10" t="s">
         <v>6</v>
       </c>
-      <c r="Q10" s="22">
+      <c r="Q10">
         <v>98.269193690481302</v>
       </c>
-      <c r="R10" s="23">
+      <c r="R10" s="22">
         <v>95.09</v>
       </c>
       <c r="T10" s="21"/>
-      <c r="U10" s="22" t="s">
+      <c r="U10" t="s">
         <v>6</v>
       </c>
-      <c r="V10" s="36">
+      <c r="V10" s="33">
         <v>98.984456578837296</v>
       </c>
-      <c r="W10" s="23">
+      <c r="W10" s="22">
         <v>95.09</v>
       </c>
       <c r="Y10" s="8"/>
       <c r="Z10" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="AA10" s="34">
+      <c r="AA10" s="31">
         <v>99.275177048739906</v>
       </c>
       <c r="AB10" s="10">
@@ -1175,56 +1174,56 @@
     </row>
     <row r="11" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C11" s="21"/>
-      <c r="D11" s="22" t="s">
+      <c r="D11" t="s">
         <v>7</v>
       </c>
-      <c r="E11" s="22">
+      <c r="E11">
         <v>96.34</v>
       </c>
-      <c r="F11" s="22" t="s">
+      <c r="F11" t="s">
         <v>21</v>
       </c>
-      <c r="G11" s="29">
+      <c r="G11" s="26">
         <v>95.09</v>
       </c>
-      <c r="H11" s="30" t="s">
+      <c r="H11" s="27" t="s">
         <v>27</v>
       </c>
       <c r="J11" s="21"/>
-      <c r="K11" s="22" t="s">
+      <c r="K11" t="s">
         <v>7</v>
       </c>
-      <c r="L11" s="22">
+      <c r="L11">
         <v>97.476847073323299</v>
       </c>
-      <c r="M11" s="23">
+      <c r="M11" s="22">
         <v>94.53</v>
       </c>
       <c r="O11" s="21"/>
-      <c r="P11" s="22" t="s">
+      <c r="P11" t="s">
         <v>7</v>
       </c>
-      <c r="Q11" s="22">
+      <c r="Q11">
         <v>97.900520199457105</v>
       </c>
-      <c r="R11" s="23">
+      <c r="R11" s="22">
         <v>93.81</v>
       </c>
       <c r="T11" s="21"/>
-      <c r="U11" s="22" t="s">
+      <c r="U11" t="s">
         <v>7</v>
       </c>
-      <c r="V11" s="36">
+      <c r="V11" s="33">
         <v>98.606619399039701</v>
       </c>
-      <c r="W11" s="23">
+      <c r="W11" s="22">
         <v>93.81</v>
       </c>
       <c r="Y11" s="8"/>
       <c r="Z11" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="AA11" s="34">
+      <c r="AA11" s="31">
         <v>98.877563424654994</v>
       </c>
       <c r="AB11" s="10">
@@ -1233,56 +1232,56 @@
     </row>
     <row r="12" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C12" s="21"/>
-      <c r="D12" s="22" t="s">
+      <c r="D12" t="s">
         <v>8</v>
       </c>
-      <c r="E12" s="22">
+      <c r="E12">
         <v>97.11</v>
       </c>
-      <c r="F12" s="22" t="s">
+      <c r="F12" t="s">
         <v>21</v>
       </c>
-      <c r="G12" s="31">
+      <c r="G12" s="28">
         <v>94.8</v>
       </c>
-      <c r="H12" s="30" t="s">
+      <c r="H12" s="27" t="s">
         <v>22</v>
       </c>
       <c r="J12" s="21"/>
-      <c r="K12" s="22" t="s">
+      <c r="K12" t="s">
         <v>8</v>
       </c>
-      <c r="L12" s="22">
+      <c r="L12">
         <v>97.977486929353006</v>
       </c>
-      <c r="M12" s="23">
+      <c r="M12" s="22">
         <v>94.66</v>
       </c>
       <c r="O12" s="21"/>
-      <c r="P12" s="22" t="s">
+      <c r="P12" t="s">
         <v>8</v>
       </c>
-      <c r="Q12" s="22">
+      <c r="Q12">
         <v>98.120668126227201</v>
       </c>
-      <c r="R12" s="23">
+      <c r="R12" s="22">
         <v>92.19</v>
       </c>
       <c r="T12" s="21"/>
-      <c r="U12" s="22" t="s">
+      <c r="U12" t="s">
         <v>8</v>
       </c>
-      <c r="V12" s="36">
+      <c r="V12" s="33">
         <v>98.554234247398796</v>
       </c>
-      <c r="W12" s="23">
+      <c r="W12" s="22">
         <v>92.34</v>
       </c>
       <c r="Y12" s="8"/>
       <c r="Z12" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="AA12" s="34">
+      <c r="AA12" s="31">
         <v>98.699674706335301</v>
       </c>
       <c r="AB12" s="10">
@@ -1293,55 +1292,55 @@
       <c r="C13" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="D13" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="E13" s="22">
+      <c r="D13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E13">
         <v>97.94</v>
       </c>
-      <c r="F13" s="22" t="s">
+      <c r="F13" t="s">
         <v>22</v>
       </c>
-      <c r="G13" s="22">
+      <c r="G13">
         <v>96.34</v>
       </c>
-      <c r="H13" s="23" t="s">
+      <c r="H13" s="22" t="s">
         <v>28</v>
       </c>
       <c r="J13" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="K13" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="L13" s="22">
+      <c r="K13" t="s">
+        <v>1</v>
+      </c>
+      <c r="L13">
         <v>98.376931659705093</v>
       </c>
-      <c r="M13" s="23">
+      <c r="M13" s="22">
         <v>95.85</v>
       </c>
       <c r="O13" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="P13" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="Q13" s="22">
+      <c r="P13" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q13">
         <v>98.378796537364295</v>
       </c>
-      <c r="R13" s="23">
+      <c r="R13" s="22">
         <v>95.85</v>
       </c>
       <c r="T13" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="U13" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="V13" s="36">
+      <c r="U13" t="s">
+        <v>1</v>
+      </c>
+      <c r="V13" s="33">
         <v>98.686403838798796</v>
       </c>
-      <c r="W13" s="23">
+      <c r="W13" s="22">
         <v>97.05</v>
       </c>
       <c r="Y13" s="8" t="s">
@@ -1350,7 +1349,7 @@
       <c r="Z13" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="AA13" s="34">
+      <c r="AA13" s="31">
         <v>98.977735045550403</v>
       </c>
       <c r="AB13" s="10">
@@ -1359,56 +1358,56 @@
     </row>
     <row r="14" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C14" s="21"/>
-      <c r="D14" s="22" t="s">
-        <v>2</v>
-      </c>
-      <c r="E14" s="22">
+      <c r="D14" t="s">
+        <v>2</v>
+      </c>
+      <c r="E14">
         <v>95.77</v>
       </c>
-      <c r="F14" s="22" t="s">
+      <c r="F14" t="s">
         <v>21</v>
       </c>
-      <c r="G14" s="22">
+      <c r="G14">
         <v>93.38</v>
       </c>
-      <c r="H14" s="23" t="s">
+      <c r="H14" s="22" t="s">
         <v>29</v>
       </c>
       <c r="J14" s="21"/>
-      <c r="K14" s="22" t="s">
-        <v>2</v>
-      </c>
-      <c r="L14" s="22">
+      <c r="K14" t="s">
+        <v>2</v>
+      </c>
+      <c r="L14">
         <v>97.088563433336503</v>
       </c>
-      <c r="M14" s="23">
+      <c r="M14" s="22">
         <v>92.9</v>
       </c>
       <c r="O14" s="21"/>
-      <c r="P14" s="22" t="s">
-        <v>2</v>
-      </c>
-      <c r="Q14" s="22">
+      <c r="P14" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q14">
         <v>98.064103972194403</v>
       </c>
-      <c r="R14" s="23">
+      <c r="R14" s="22">
         <v>93.47</v>
       </c>
       <c r="T14" s="21"/>
-      <c r="U14" s="22" t="s">
-        <v>2</v>
-      </c>
-      <c r="V14" s="36">
+      <c r="U14" t="s">
+        <v>2</v>
+      </c>
+      <c r="V14" s="33">
         <v>98.748524920891498</v>
       </c>
-      <c r="W14" s="23">
+      <c r="W14" s="22">
         <v>93.47</v>
       </c>
       <c r="Y14" s="8"/>
       <c r="Z14" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="AA14" s="34">
+      <c r="AA14" s="31">
         <v>99.020127901968905</v>
       </c>
       <c r="AB14" s="10">
@@ -1419,55 +1418,55 @@
       <c r="C15" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="D15" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="E15" s="22">
+      <c r="D15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E15">
         <v>94.02</v>
       </c>
-      <c r="F15" s="22" t="s">
+      <c r="F15" t="s">
         <v>21</v>
       </c>
-      <c r="G15" s="22">
+      <c r="G15">
         <v>88.31</v>
       </c>
-      <c r="H15" s="23" t="s">
+      <c r="H15" s="22" t="s">
         <v>22</v>
       </c>
       <c r="J15" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="K15" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="L15" s="22">
+      <c r="K15" t="s">
+        <v>3</v>
+      </c>
+      <c r="L15">
         <v>96.350895844665303</v>
       </c>
-      <c r="M15" s="23">
+      <c r="M15" s="22">
         <v>91.39</v>
       </c>
       <c r="O15" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="P15" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q15" s="22">
+      <c r="P15" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q15">
         <v>97.235785607012502</v>
       </c>
-      <c r="R15" s="23">
+      <c r="R15" s="22">
         <v>92.12</v>
       </c>
       <c r="T15" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="U15" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="V15" s="36">
+      <c r="U15" t="s">
+        <v>3</v>
+      </c>
+      <c r="V15" s="33">
         <v>97.5323644666679</v>
       </c>
-      <c r="W15" s="23">
+      <c r="W15" s="22">
         <v>92.12</v>
       </c>
       <c r="Y15" s="8" t="s">
@@ -1476,7 +1475,7 @@
       <c r="Z15" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="AA15" s="34">
+      <c r="AA15" s="31">
         <v>98.405691077923606</v>
       </c>
       <c r="AB15" s="10">
@@ -1485,56 +1484,56 @@
     </row>
     <row r="16" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C16" s="21"/>
-      <c r="D16" s="22" t="s">
-        <v>4</v>
-      </c>
-      <c r="E16" s="22">
+      <c r="D16" t="s">
+        <v>4</v>
+      </c>
+      <c r="E16">
         <v>92.38</v>
       </c>
-      <c r="F16" s="22" t="s">
+      <c r="F16" t="s">
         <v>21</v>
       </c>
-      <c r="G16" s="29">
+      <c r="G16" s="26">
         <v>89.25</v>
       </c>
-      <c r="H16" s="30" t="s">
+      <c r="H16" s="27" t="s">
         <v>22</v>
       </c>
       <c r="J16" s="21"/>
-      <c r="K16" s="22" t="s">
-        <v>4</v>
-      </c>
-      <c r="L16" s="22">
+      <c r="K16" t="s">
+        <v>4</v>
+      </c>
+      <c r="L16">
         <v>94.694633144244506</v>
       </c>
-      <c r="M16" s="23">
+      <c r="M16" s="22">
         <v>87.56</v>
       </c>
       <c r="O16" s="21"/>
-      <c r="P16" s="22" t="s">
-        <v>4</v>
-      </c>
-      <c r="Q16" s="22">
+      <c r="P16" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q16">
         <v>96.515280236400699</v>
       </c>
-      <c r="R16" s="23">
+      <c r="R16" s="22">
         <v>87.03</v>
       </c>
       <c r="T16" s="21"/>
-      <c r="U16" s="22" t="s">
-        <v>4</v>
-      </c>
-      <c r="V16" s="36">
+      <c r="U16" t="s">
+        <v>4</v>
+      </c>
+      <c r="V16" s="33">
         <v>97.082873928417598</v>
       </c>
-      <c r="W16" s="23">
+      <c r="W16" s="22">
         <v>87.84</v>
       </c>
       <c r="Y16" s="8"/>
       <c r="Z16" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="AA16" s="34">
+      <c r="AA16" s="31">
         <v>97.764375291161798</v>
       </c>
       <c r="AB16" s="10">
@@ -1545,55 +1544,55 @@
       <c r="C17" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="D17" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="E17" s="22">
+      <c r="D17" t="s">
+        <v>1</v>
+      </c>
+      <c r="E17">
         <v>87.81</v>
       </c>
-      <c r="F17" s="22" t="s">
+      <c r="F17" t="s">
         <v>18</v>
       </c>
-      <c r="G17" s="22">
+      <c r="G17">
         <v>81.98</v>
       </c>
-      <c r="H17" s="23" t="s">
+      <c r="H17" s="22" t="s">
         <v>28</v>
       </c>
       <c r="J17" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="K17" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="L17" s="22">
+      <c r="K17" t="s">
+        <v>1</v>
+      </c>
+      <c r="L17">
         <v>91.147926522397597</v>
       </c>
-      <c r="M17" s="23">
+      <c r="M17" s="22">
         <v>85.33</v>
       </c>
       <c r="O17" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="P17" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="Q17" s="22">
+      <c r="P17" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q17">
         <v>94.654390676422494</v>
       </c>
-      <c r="R17" s="23">
+      <c r="R17" s="22">
         <v>85.98</v>
       </c>
       <c r="T17" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="U17" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="V17" s="36">
+      <c r="U17" t="s">
+        <v>1</v>
+      </c>
+      <c r="V17" s="33">
         <v>94.809557800717499</v>
       </c>
-      <c r="W17" s="23">
+      <c r="W17" s="22">
         <v>90.25</v>
       </c>
       <c r="Y17" s="8" t="s">
@@ -1602,7 +1601,7 @@
       <c r="Z17" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="AA17" s="34">
+      <c r="AA17" s="31">
         <v>95.541206383771197</v>
       </c>
       <c r="AB17" s="10">
@@ -1611,56 +1610,56 @@
     </row>
     <row r="18" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C18" s="21"/>
-      <c r="D18" s="22" t="s">
-        <v>2</v>
-      </c>
-      <c r="E18" s="22">
+      <c r="D18" t="s">
+        <v>2</v>
+      </c>
+      <c r="E18">
         <v>75.17</v>
       </c>
-      <c r="F18" s="22" t="s">
+      <c r="F18" t="s">
         <v>17</v>
       </c>
-      <c r="G18" s="22">
+      <c r="G18">
         <v>75.06</v>
       </c>
-      <c r="H18" s="23" t="s">
+      <c r="H18" s="22" t="s">
         <v>28</v>
       </c>
       <c r="J18" s="21"/>
-      <c r="K18" s="22" t="s">
-        <v>2</v>
-      </c>
-      <c r="L18" s="22">
+      <c r="K18" t="s">
+        <v>2</v>
+      </c>
+      <c r="L18">
         <v>81.629911824847895</v>
       </c>
-      <c r="M18" s="23">
+      <c r="M18" s="22">
         <v>69.34</v>
       </c>
       <c r="O18" s="21"/>
-      <c r="P18" s="22" t="s">
-        <v>2</v>
-      </c>
-      <c r="Q18" s="22">
+      <c r="P18" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q18">
         <v>86.487738453020896</v>
       </c>
-      <c r="R18" s="23">
+      <c r="R18" s="22">
         <v>71.72</v>
       </c>
       <c r="T18" s="21"/>
-      <c r="U18" s="22" t="s">
-        <v>2</v>
-      </c>
-      <c r="V18" s="36">
+      <c r="U18" t="s">
+        <v>2</v>
+      </c>
+      <c r="V18" s="33">
         <v>88.224547339506898</v>
       </c>
-      <c r="W18" s="23">
+      <c r="W18" s="22">
         <v>76.87</v>
       </c>
       <c r="Y18" s="8"/>
       <c r="Z18" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="AA18" s="34">
+      <c r="AA18" s="31">
         <v>90.931657961583497</v>
       </c>
       <c r="AB18" s="10">
@@ -1669,56 +1668,56 @@
     </row>
     <row r="19" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C19" s="21"/>
-      <c r="D19" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="E19" s="22">
+      <c r="D19" t="s">
+        <v>3</v>
+      </c>
+      <c r="E19">
         <v>73.91</v>
       </c>
-      <c r="F19" s="22" t="s">
+      <c r="F19" t="s">
         <v>16</v>
       </c>
-      <c r="G19" s="22">
+      <c r="G19">
         <v>65.31</v>
       </c>
-      <c r="H19" s="23" t="s">
+      <c r="H19" s="22" t="s">
         <v>29</v>
       </c>
       <c r="J19" s="21"/>
-      <c r="K19" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="L19" s="22">
+      <c r="K19" t="s">
+        <v>3</v>
+      </c>
+      <c r="L19">
         <v>73.341941359279204</v>
       </c>
-      <c r="M19" s="23">
+      <c r="M19" s="22">
         <v>59.19</v>
       </c>
       <c r="O19" s="21"/>
-      <c r="P19" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q19" s="22">
+      <c r="P19" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q19">
         <v>75.483002967830302</v>
       </c>
-      <c r="R19" s="23">
+      <c r="R19" s="22">
         <v>59.83</v>
       </c>
       <c r="T19" s="21"/>
-      <c r="U19" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="V19" s="36">
+      <c r="U19" t="s">
+        <v>3</v>
+      </c>
+      <c r="V19" s="33">
         <v>78.653498543930596</v>
       </c>
-      <c r="W19" s="23">
+      <c r="W19" s="22">
         <v>67.599999999999994</v>
       </c>
       <c r="Y19" s="8"/>
       <c r="Z19" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="AA19" s="34">
+      <c r="AA19" s="31">
         <v>82.154690212955103</v>
       </c>
       <c r="AB19" s="10">
@@ -1727,56 +1726,56 @@
     </row>
     <row r="20" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C20" s="21"/>
-      <c r="D20" s="22" t="s">
-        <v>4</v>
-      </c>
-      <c r="E20" s="22">
+      <c r="D20" t="s">
+        <v>4</v>
+      </c>
+      <c r="E20">
         <v>67.52</v>
       </c>
-      <c r="F20" s="22" t="s">
+      <c r="F20" t="s">
         <v>16</v>
       </c>
-      <c r="G20" s="22">
+      <c r="G20">
         <v>56.03</v>
       </c>
-      <c r="H20" s="23" t="s">
+      <c r="H20" s="22" t="s">
         <v>30</v>
       </c>
       <c r="J20" s="21"/>
-      <c r="K20" s="22" t="s">
-        <v>4</v>
-      </c>
-      <c r="L20" s="22">
+      <c r="K20" t="s">
+        <v>4</v>
+      </c>
+      <c r="L20">
         <v>70.907524436112993</v>
       </c>
-      <c r="M20" s="23">
+      <c r="M20" s="22">
         <v>52.44</v>
       </c>
       <c r="O20" s="21"/>
-      <c r="P20" s="22" t="s">
-        <v>4</v>
-      </c>
-      <c r="Q20" s="22">
+      <c r="P20" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q20">
         <v>72.685883512840306</v>
       </c>
-      <c r="R20" s="23">
+      <c r="R20" s="22">
         <v>52.57</v>
       </c>
       <c r="T20" s="21"/>
-      <c r="U20" s="22" t="s">
-        <v>4</v>
-      </c>
-      <c r="V20" s="36">
+      <c r="U20" t="s">
+        <v>4</v>
+      </c>
+      <c r="V20" s="33">
         <v>73.378405689436605</v>
       </c>
-      <c r="W20" s="23">
+      <c r="W20" s="22">
         <v>60.65</v>
       </c>
       <c r="Y20" s="8"/>
       <c r="Z20" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="AA20" s="34">
+      <c r="AA20" s="31">
         <v>73.362430753735097</v>
       </c>
       <c r="AB20" s="10">
@@ -1787,55 +1786,55 @@
       <c r="C21" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="D21" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="E21" s="22">
+      <c r="D21" t="s">
+        <v>1</v>
+      </c>
+      <c r="E21">
         <v>98.21</v>
       </c>
-      <c r="F21" s="22" t="s">
+      <c r="F21" t="s">
         <v>20</v>
       </c>
-      <c r="G21" s="22">
+      <c r="G21">
         <v>95.54</v>
       </c>
-      <c r="H21" s="23" t="s">
+      <c r="H21" s="22" t="s">
         <v>31</v>
       </c>
       <c r="J21" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="K21" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="L21" s="22">
+      <c r="K21" t="s">
+        <v>1</v>
+      </c>
+      <c r="L21">
         <v>98.812157448928701</v>
       </c>
-      <c r="M21" s="23">
+      <c r="M21" s="22">
         <v>96.44</v>
       </c>
       <c r="O21" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="P21" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="Q21" s="22">
+      <c r="P21" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q21">
         <v>99.257587456197697</v>
       </c>
-      <c r="R21" s="23">
+      <c r="R21" s="22">
         <v>96.59</v>
       </c>
       <c r="T21" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="U21" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="V21" s="36">
+      <c r="U21" t="s">
+        <v>1</v>
+      </c>
+      <c r="V21" s="33">
         <v>99.405747339635894</v>
       </c>
-      <c r="W21" s="23">
+      <c r="W21" s="22">
         <v>96.73</v>
       </c>
       <c r="Y21" s="8" t="s">
@@ -1844,7 +1843,7 @@
       <c r="Z21" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="AA21" s="34">
+      <c r="AA21" s="31">
         <v>99.406080246848006</v>
       </c>
       <c r="AB21" s="10">
@@ -1853,56 +1852,56 @@
     </row>
     <row r="22" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C22" s="21"/>
-      <c r="D22" s="22" t="s">
-        <v>2</v>
-      </c>
-      <c r="E22" s="22">
+      <c r="D22" t="s">
+        <v>2</v>
+      </c>
+      <c r="E22">
         <v>97.87</v>
       </c>
-      <c r="F22" s="22" t="s">
+      <c r="F22" t="s">
         <v>20</v>
       </c>
-      <c r="G22" s="22">
+      <c r="G22">
         <v>97.97</v>
       </c>
-      <c r="H22" s="23" t="s">
+      <c r="H22" s="22" t="s">
         <v>27</v>
       </c>
       <c r="J22" s="21"/>
-      <c r="K22" s="22" t="s">
-        <v>2</v>
-      </c>
-      <c r="L22" s="22">
+      <c r="K22" t="s">
+        <v>2</v>
+      </c>
+      <c r="L22">
         <v>98.704544168208102</v>
       </c>
-      <c r="M22" s="23">
+      <c r="M22" s="22">
         <v>97.13</v>
       </c>
       <c r="O22" s="21"/>
-      <c r="P22" s="22" t="s">
-        <v>2</v>
-      </c>
-      <c r="Q22" s="22">
+      <c r="P22" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q22">
         <v>99.145841399601693</v>
       </c>
-      <c r="R22" s="23">
+      <c r="R22" s="22">
         <v>98.12</v>
       </c>
       <c r="T22" s="21"/>
-      <c r="U22" s="22" t="s">
-        <v>2</v>
-      </c>
-      <c r="V22" s="36">
+      <c r="U22" t="s">
+        <v>2</v>
+      </c>
+      <c r="V22" s="33">
         <v>99.145841399601693</v>
       </c>
-      <c r="W22" s="23">
+      <c r="W22" s="22">
         <v>98.12</v>
       </c>
       <c r="Y22" s="8"/>
       <c r="Z22" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="AA22" s="34">
+      <c r="AA22" s="31">
         <v>99.420888729189102</v>
       </c>
       <c r="AB22" s="10">
@@ -1911,56 +1910,56 @@
     </row>
     <row r="23" spans="3:28" x14ac:dyDescent="0.2">
       <c r="C23" s="21"/>
-      <c r="D23" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="E23" s="22">
+      <c r="D23" t="s">
+        <v>3</v>
+      </c>
+      <c r="E23">
         <v>96.66</v>
       </c>
-      <c r="F23" s="22" t="s">
+      <c r="F23" t="s">
         <v>20</v>
       </c>
-      <c r="G23" s="29">
+      <c r="G23" s="26">
         <v>91.22</v>
       </c>
-      <c r="H23" s="30" t="s">
+      <c r="H23" s="27" t="s">
         <v>29</v>
       </c>
       <c r="J23" s="21"/>
-      <c r="K23" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="L23" s="22">
+      <c r="K23" t="s">
+        <v>3</v>
+      </c>
+      <c r="L23">
         <v>98.406471705325202</v>
       </c>
-      <c r="M23" s="23">
+      <c r="M23" s="22">
         <v>91.24</v>
       </c>
       <c r="O23" s="21"/>
-      <c r="P23" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q23" s="22">
+      <c r="P23" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q23">
         <v>98.837336777703896</v>
       </c>
-      <c r="R23" s="23">
+      <c r="R23" s="22">
         <v>91.06</v>
       </c>
       <c r="T23" s="21"/>
-      <c r="U23" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="V23" s="36">
+      <c r="U23" t="s">
+        <v>3</v>
+      </c>
+      <c r="V23" s="33">
         <v>99.415675914599205</v>
       </c>
-      <c r="W23" s="23">
+      <c r="W23" s="22">
         <v>91.2</v>
       </c>
       <c r="Y23" s="8"/>
       <c r="Z23" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="AA23" s="34">
+      <c r="AA23" s="31">
         <v>99.561389670192</v>
       </c>
       <c r="AB23" s="10">
@@ -1968,57 +1967,57 @@
       </c>
     </row>
     <row r="24" spans="3:28" x14ac:dyDescent="0.2">
-      <c r="C24" s="24"/>
-      <c r="D24" s="25" t="s">
-        <v>4</v>
-      </c>
-      <c r="E24" s="25">
+      <c r="C24" s="23"/>
+      <c r="D24" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="E24" s="24">
         <v>95.99</v>
       </c>
-      <c r="F24" s="25" t="s">
+      <c r="F24" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="G24" s="32">
+      <c r="G24" s="29">
         <v>86.35</v>
       </c>
-      <c r="H24" s="33" t="s">
+      <c r="H24" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="J24" s="24"/>
-      <c r="K24" s="25" t="s">
-        <v>4</v>
-      </c>
-      <c r="L24" s="25">
+      <c r="J24" s="23"/>
+      <c r="K24" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="L24" s="24">
         <v>97.562728083059596</v>
       </c>
-      <c r="M24" s="26">
+      <c r="M24" s="25">
         <v>86.58</v>
       </c>
-      <c r="O24" s="24"/>
-      <c r="P24" s="25" t="s">
-        <v>4</v>
-      </c>
-      <c r="Q24" s="25">
+      <c r="O24" s="23"/>
+      <c r="P24" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q24" s="24">
         <v>98.570849475026904</v>
       </c>
-      <c r="R24" s="26">
+      <c r="R24" s="25">
         <v>87.33</v>
       </c>
-      <c r="T24" s="24"/>
-      <c r="U24" s="25" t="s">
-        <v>4</v>
-      </c>
-      <c r="V24" s="37">
+      <c r="T24" s="23"/>
+      <c r="U24" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="V24" s="34">
         <v>99.284894815269993</v>
       </c>
-      <c r="W24" s="26">
+      <c r="W24" s="25">
         <v>87.6</v>
       </c>
       <c r="Y24" s="11"/>
       <c r="Z24" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="AA24" s="35">
+      <c r="AA24" s="32">
         <v>99.429148404313693</v>
       </c>
       <c r="AB24" s="13">
@@ -2108,7 +2107,7 @@
       <c r="K29" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="L29" s="34">
+      <c r="L29" s="31">
         <v>99.291809243086405</v>
       </c>
       <c r="M29" s="10">
@@ -2120,7 +2119,7 @@
       <c r="P29" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="Q29" s="34">
+      <c r="Q29" s="31">
         <v>99.286751324742198</v>
       </c>
       <c r="R29" s="10">
@@ -2132,7 +2131,7 @@
       <c r="U29" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="V29" s="34">
+      <c r="V29" s="31">
         <v>99.437427660605707</v>
       </c>
       <c r="W29" s="10">
@@ -2156,7 +2155,7 @@
       <c r="K30" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="L30" s="34">
+      <c r="L30" s="31">
         <v>99.718430602154697</v>
       </c>
       <c r="M30" s="10">
@@ -2166,7 +2165,7 @@
       <c r="P30" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="Q30" s="34">
+      <c r="Q30" s="31">
         <v>99.727306186636298</v>
       </c>
       <c r="R30" s="10">
@@ -2176,7 +2175,7 @@
       <c r="U30" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="V30" s="34">
+      <c r="V30" s="31">
         <v>99.863658225465798</v>
       </c>
       <c r="W30" s="10">
@@ -2198,7 +2197,7 @@
       <c r="K31" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="L31" s="34">
+      <c r="L31" s="31">
         <v>99.557056500397493</v>
       </c>
       <c r="M31" s="10">
@@ -2208,7 +2207,7 @@
       <c r="P31" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="Q31" s="34">
+      <c r="Q31" s="31">
         <v>99.557485453805995</v>
       </c>
       <c r="R31" s="10">
@@ -2218,7 +2217,7 @@
       <c r="U31" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="V31" s="34">
+      <c r="V31" s="31">
         <v>99.562562667966205</v>
       </c>
       <c r="W31" s="10">
@@ -2240,7 +2239,7 @@
       <c r="K32" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="L32" s="34">
+      <c r="L32" s="31">
         <v>99.278134262279593</v>
       </c>
       <c r="M32" s="10">
@@ -2250,7 +2249,7 @@
       <c r="P32" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="Q32" s="34">
+      <c r="Q32" s="31">
         <v>99.419274106080806</v>
       </c>
       <c r="R32" s="10">
@@ -2260,7 +2259,7 @@
       <c r="U32" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="V32" s="34">
+      <c r="V32" s="31">
         <v>99.435311533732104</v>
       </c>
       <c r="W32" s="10">
@@ -2282,7 +2281,7 @@
       <c r="K33" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="L33" s="34">
+      <c r="L33" s="31">
         <v>99.695824357606298</v>
       </c>
       <c r="M33" s="10">
@@ -2292,7 +2291,7 @@
       <c r="P33" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="Q33" s="34">
+      <c r="Q33" s="31">
         <v>99.695824357606298</v>
       </c>
       <c r="R33" s="10">
@@ -2302,7 +2301,7 @@
       <c r="U33" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="V33" s="34">
+      <c r="V33" s="31">
         <v>99.5456400230876</v>
       </c>
       <c r="W33" s="10">
@@ -2324,7 +2323,7 @@
       <c r="K34" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="L34" s="34">
+      <c r="L34" s="31">
         <v>99.419140829703693</v>
       </c>
       <c r="M34" s="10">
@@ -2334,7 +2333,7 @@
       <c r="P34" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="Q34" s="34">
+      <c r="Q34" s="31">
         <v>99.562345704744303</v>
       </c>
       <c r="R34" s="10">
@@ -2344,7 +2343,7 @@
       <c r="U34" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="V34" s="34">
+      <c r="V34" s="31">
         <v>99.562345704744303</v>
       </c>
       <c r="W34" s="10">
@@ -2366,7 +2365,7 @@
       <c r="K35" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="L35" s="34">
+      <c r="L35" s="31">
         <v>99.016179267225297</v>
       </c>
       <c r="M35" s="10">
@@ -2376,7 +2375,7 @@
       <c r="P35" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="Q35" s="34">
+      <c r="Q35" s="31">
         <v>99.154784846329704</v>
       </c>
       <c r="R35" s="10">
@@ -2386,7 +2385,7 @@
       <c r="U35" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="V35" s="34">
+      <c r="V35" s="31">
         <v>99.297085790328296</v>
       </c>
       <c r="W35" s="10">
@@ -2408,7 +2407,7 @@
       <c r="K36" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="L36" s="34">
+      <c r="L36" s="31">
         <v>98.844172789062895</v>
       </c>
       <c r="M36" s="10">
@@ -2418,7 +2417,7 @@
       <c r="P36" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="Q36" s="34">
+      <c r="Q36" s="31">
         <v>98.8442690766353</v>
       </c>
       <c r="R36" s="10">
@@ -2428,7 +2427,7 @@
       <c r="U36" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="V36" s="34">
+      <c r="V36" s="31">
         <v>98.988531710822997</v>
       </c>
       <c r="W36" s="10">
@@ -2452,7 +2451,7 @@
       <c r="K37" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="L37" s="34">
+      <c r="L37" s="31">
         <v>98.832260982766698</v>
       </c>
       <c r="M37" s="10">
@@ -2464,7 +2463,7 @@
       <c r="P37" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="Q37" s="34">
+      <c r="Q37" s="31">
         <v>99.412022746388999</v>
       </c>
       <c r="R37" s="10">
@@ -2476,7 +2475,7 @@
       <c r="U37" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="V37" s="34">
+      <c r="V37" s="31">
         <v>99.559884559884594</v>
       </c>
       <c r="W37" s="10">
@@ -2500,7 +2499,7 @@
       <c r="K38" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="L38" s="34">
+      <c r="L38" s="31">
         <v>99.321683383310898</v>
       </c>
       <c r="M38" s="10">
@@ -2510,7 +2509,7 @@
       <c r="P38" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="Q38" s="34">
+      <c r="Q38" s="31">
         <v>99.444209125115506</v>
       </c>
       <c r="R38" s="10">
@@ -2520,7 +2519,7 @@
       <c r="U38" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="V38" s="34">
+      <c r="V38" s="31">
         <v>99.714977597725394</v>
       </c>
       <c r="W38" s="10">
@@ -2544,7 +2543,7 @@
       <c r="K39" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="L39" s="34">
+      <c r="L39" s="31">
         <v>98.6943123585839</v>
       </c>
       <c r="M39" s="10">
@@ -2556,7 +2555,7 @@
       <c r="P39" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="Q39" s="34">
+      <c r="Q39" s="31">
         <v>98.991989399144998</v>
       </c>
       <c r="R39" s="10">
@@ -2568,7 +2567,7 @@
       <c r="U39" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="V39" s="34">
+      <c r="V39" s="31">
         <v>99.415003006576299</v>
       </c>
       <c r="W39" s="10">
@@ -2592,7 +2591,7 @@
       <c r="K40" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="L40" s="34">
+      <c r="L40" s="31">
         <v>98.460603284465705</v>
       </c>
       <c r="M40" s="10">
@@ -2602,7 +2601,7 @@
       <c r="P40" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="Q40" s="34">
+      <c r="Q40" s="31">
         <v>99.015448244999703</v>
       </c>
       <c r="R40" s="10">
@@ -2612,7 +2611,7 @@
       <c r="U40" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="V40" s="34">
+      <c r="V40" s="31">
         <v>99.165946413137405</v>
       </c>
       <c r="W40" s="10">
@@ -2636,7 +2635,7 @@
       <c r="K41" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="L41" s="34">
+      <c r="L41" s="31">
         <v>96.1293845221943</v>
       </c>
       <c r="M41" s="10">
@@ -2648,7 +2647,7 @@
       <c r="P41" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="Q41" s="34">
+      <c r="Q41" s="31">
         <v>96.582893546840396</v>
       </c>
       <c r="R41" s="10">
@@ -2660,7 +2659,7 @@
       <c r="U41" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="V41" s="34">
+      <c r="V41" s="31">
         <v>96.582893546840396</v>
       </c>
       <c r="W41" s="10">
@@ -2684,7 +2683,7 @@
       <c r="K42" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="L42" s="34">
+      <c r="L42" s="31">
         <v>91.423141791576597</v>
       </c>
       <c r="M42" s="10">
@@ -2694,7 +2693,7 @@
       <c r="P42" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="Q42" s="34">
+      <c r="Q42" s="31">
         <v>93.302766388734199</v>
       </c>
       <c r="R42" s="10">
@@ -2704,7 +2703,7 @@
       <c r="U42" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="V42" s="34">
+      <c r="V42" s="31">
         <v>93.442317389910599</v>
       </c>
       <c r="W42" s="10">
@@ -2726,7 +2725,7 @@
       <c r="K43" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="L43" s="34">
+      <c r="L43" s="31">
         <v>82.728818217052606</v>
       </c>
       <c r="M43" s="10">
@@ -2736,7 +2735,7 @@
       <c r="P43" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="Q43" s="34">
+      <c r="Q43" s="31">
         <v>82.880996223891501</v>
       </c>
       <c r="R43" s="10">
@@ -2746,7 +2745,7 @@
       <c r="U43" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="V43" s="34">
+      <c r="V43" s="31">
         <v>82.052981256516603</v>
       </c>
       <c r="W43" s="10">
@@ -2768,7 +2767,7 @@
       <c r="K44" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="L44" s="34">
+      <c r="L44" s="31">
         <v>73.576345245828605</v>
       </c>
       <c r="M44" s="10">
@@ -2778,7 +2777,7 @@
       <c r="P44" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="Q44" s="34">
+      <c r="Q44" s="31">
         <v>73.234084342379603</v>
       </c>
       <c r="R44" s="10">
@@ -2788,7 +2787,7 @@
       <c r="U44" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="V44" s="34">
+      <c r="V44" s="31">
         <v>73.654970760233894</v>
       </c>
       <c r="W44" s="10">
@@ -2812,7 +2811,7 @@
       <c r="K45" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="L45" s="34">
+      <c r="L45" s="31">
         <v>99.554222512587998</v>
       </c>
       <c r="M45" s="10">
@@ -2824,7 +2823,7 @@
       <c r="P45" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="Q45" s="34">
+      <c r="Q45" s="31">
         <v>99.554222512587998</v>
       </c>
       <c r="R45" s="10">
@@ -2836,7 +2835,7 @@
       <c r="U45" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="V45" s="34">
+      <c r="V45" s="31">
         <v>99.554222512587998</v>
       </c>
       <c r="W45" s="10">
@@ -2860,7 +2859,7 @@
       <c r="K46" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="L46" s="34">
+      <c r="L46" s="31">
         <v>99.572447336422499</v>
       </c>
       <c r="M46" s="10">
@@ -2870,7 +2869,7 @@
       <c r="P46" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="Q46" s="34">
+      <c r="Q46" s="31">
         <v>99.717387269254502</v>
       </c>
       <c r="R46" s="10">
@@ -2880,7 +2879,7 @@
       <c r="U46" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="V46" s="34">
+      <c r="V46" s="31">
         <v>99.858680307609802</v>
       </c>
       <c r="W46" s="10">
@@ -2902,7 +2901,7 @@
       <c r="K47" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="L47" s="34">
+      <c r="L47" s="31">
         <v>99.561389670192</v>
       </c>
       <c r="M47" s="10">
@@ -2912,7 +2911,7 @@
       <c r="P47" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="Q47" s="34">
+      <c r="Q47" s="31">
         <v>99.561389670192</v>
       </c>
       <c r="R47" s="10">
@@ -2922,7 +2921,7 @@
       <c r="U47" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="V47" s="34">
+      <c r="V47" s="31">
         <v>99.561389670192</v>
       </c>
       <c r="W47" s="10">
@@ -2944,7 +2943,7 @@
       <c r="K48" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="L48" s="35">
+      <c r="L48" s="32">
         <v>99.719868173258007</v>
       </c>
       <c r="M48" s="13">
@@ -2954,7 +2953,7 @@
       <c r="P48" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="Q48" s="35">
+      <c r="Q48" s="32">
         <v>99.719868173258007</v>
       </c>
       <c r="R48" s="13">
@@ -2964,7 +2963,7 @@
       <c r="U48" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="V48" s="35">
+      <c r="V48" s="32">
         <v>99.719868173258007</v>
       </c>
       <c r="W48" s="13">

</xml_diff>

<commit_message>
Tested two training set sizes and removed the rng seed
</commit_message>
<xml_diff>
--- a/results/validate_results.xlsx
+++ b/results/validate_results.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emily/Library/CloudStorage/GoogleDrive-u0835353@gcloud.utah.edu/.shortcut-targets-by-id/109kT4myKnMujFK8ni-DWM3IQ1FnMmvXr/EYANG/BCI Project/FWHT_FeatureExtract/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A92D5BD-335D-864E-AF1A-DFF409ED678C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01319369-28C2-DA40-83EE-8E81BFF65B88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16240" xr2:uid="{AFAE147A-AF5E-4547-B045-936377B9E7D9}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16240" activeTab="1" xr2:uid="{AFAE147A-AF5E-4547-B045-936377B9E7D9}"/>
   </bookViews>
   <sheets>
     <sheet name="baseline_slidingWindow" sheetId="1" r:id="rId1"/>
+    <sheet name="baseline+changes" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="51">
   <si>
     <t>Easy1</t>
   </si>
@@ -174,6 +175,21 @@
   </si>
   <si>
     <t>Euclidean</t>
+  </si>
+  <si>
+    <t>Most similar to  Meng implementation</t>
+  </si>
+  <si>
+    <t>Add Manhattan</t>
+  </si>
+  <si>
+    <t>Add Norm</t>
+  </si>
+  <si>
+    <t>Add Shift 12</t>
+  </si>
+  <si>
+    <t>Add Shift 12/Manhattan</t>
   </si>
 </sst>
 </file>
@@ -381,6 +397,236 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>12700</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>12700</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>118110</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{26B2B5A9-0E7F-EB4C-A87D-7183E350414F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:srcRect l="10131" t="3843" r="8170" b="7183"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="838200" y="431800"/>
+          <a:ext cx="8255000" cy="4969510"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>12700</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>12700</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>819888</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FE71074D-FF08-A7D3-0757-641852C330F3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:srcRect l="9967" t="4139" r="8660" b="6886"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9918700" y="419100"/>
+          <a:ext cx="8236688" cy="4978400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>12700</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>12700</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>12700</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>65740</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9931A778-022B-D7B9-C63E-A734D146D0C1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:srcRect l="10131" t="4433" r="8333" b="7479"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="838200" y="5905500"/>
+          <a:ext cx="8255000" cy="4929840"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>203199</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>25400</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>74878</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6F5D8167-B656-14CD-055B-6289C22710BC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:srcRect l="9805" t="4434" r="8496" b="7183"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9906000" y="5892799"/>
+          <a:ext cx="8280400" cy="4951679"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>12699</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>685800</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>11558</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{57E49203-3614-F8FC-0333-A964B8459FB5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:srcRect l="9968" t="3547" r="8170" b="7480"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18986500" y="3467099"/>
+          <a:ext cx="8115300" cy="4875659"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2987,4 +3233,36 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CAE1AAD-DD72-3143-A474-C213381992BB}">
+  <dimension ref="B2:X29"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="2" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B2" t="s">
+        <v>46</v>
+      </c>
+      <c r="M2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="X17" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="29" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B29" t="s">
+        <v>48</v>
+      </c>
+      <c r="M29" t="s">
+        <v>49</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>